<commit_message>
Manifiesto 2026: hojas SUSTITUIDAS por las renovadas (Talavera, Grinon)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/manifiesto_hojas_2026.xlsx
+++ b/docs/manifiesto_hojas_2026.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E8E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -77,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -95,6 +100,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2375,9 +2383,9 @@
           <t>HE-2026-0029</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2424,7 +2432,8 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>PARA TI · ¿versión o distinta?: La de enero es proyecto de ascensor (7.500) + subvención accesibilidad (1.980 fijo); la de septiembre es solo subvenciones accesibilidad a éxito (3,5%) + documentación técnica 1.980, sin proyecto: no se sabe si sustituye a la de enero (la comunidad renunció al proyecto) o es un encargo nuevo de subvención; ninguna firmada.</t>
+          <t>SUSTITUIDA: En enero pidieron precio y se mandó todo junto; en septiembre retomaron y pidieron las hojas renovadas (Mónica).
+sustituida por: HE-2026-0739, HE-2026-0740</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2914,9 +2923,9 @@
           <t>HE-2026-0038</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2961,7 +2970,12 @@
           <t>1ceIPIoGauQodjqLaU66SYkMj51NLdoKAonVstpXhQl8</t>
         </is>
       </c>
-      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: Mismo patrón y mismo administrador que Joaquina Santander 37 (aplicado por analogía; confirmar).
+sustituida por: HE-2026-0749, HE-2026-0750</t>
+        </is>
+      </c>
       <c r="R39" s="2" t="inlineStr"/>
       <c r="S39" s="4" t="inlineStr"/>
     </row>
@@ -5143,7 +5157,7 @@
           <t>HE-2026-0072</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>ANULADA</t>
         </is>
@@ -17600,7 +17614,7 @@
           <t>HE-2026-0271</t>
         </is>
       </c>
-      <c r="B272" s="6" t="inlineStr">
+      <c r="B272" s="7" t="inlineStr">
         <is>
           <t>ANULADA</t>
         </is>
@@ -21198,9 +21212,9 @@
           <t>HE-2026-0330</t>
         </is>
       </c>
-      <c r="B331" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B331" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
@@ -21253,8 +21267,9 @@
       </c>
       <c r="Q331" s="2" t="inlineStr">
         <is>
-          <t>versiones (leído): Las dos de 25-abr son el mismo Google Doc (mismo id) renombrado, proyecto de ascensor más subvenciones; la de 18-sep queda aparte porque solo trae subvenciones con IEE/CEE, sin proyecto, y no se sabe si sustituye a la de abril o es un encargo nuevo.
-versiones (leído): Las dos de 25-abr son el mismo Google Doc (mismo id) renombrado, proyecto de ascensor más subvenciones; la de 18-sep queda aparte porque solo trae subvenciones con IEE/CEE, sin proyecto, y no se sabe si sustituye a la de abril o es un encargo nuevo.</t>
+          <t>SUSTITUIDA: Mismo caso: renovadas en septiembre en el formato actual (Mónica).
+SUSTITUIDA: Mismo caso: renovadas en septiembre en el formato actual (Mónica).
+sustituida por: HE-2026-0734, HE-2026-0735</t>
         </is>
       </c>
       <c r="R331" s="2" t="inlineStr"/>
@@ -22257,9 +22272,9 @@
           <t>HE-2026-0347</t>
         </is>
       </c>
-      <c r="B348" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B348" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
@@ -22306,7 +22321,8 @@
       </c>
       <c r="Q348" s="2" t="inlineStr">
         <is>
-          <t>PARA TI · ¿versión o distinta?: La del 05-05 es proyecto de ascensor + subvenciones (nº 2026/04/056); las dos del 25-09 son solo subvenciones a éxito + doc. técnica 1.980, una de accesibilidad y otra de accesibilidad + eficiencia energética (más libro del edificio), con la misma fecha: parecen alternativas enviadas a la vez y no se sabe si sustituyen a la de mayo o son un encargo nuevo de subvención.</t>
+          <t>SUSTITUIDA: Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).
+sustituida por: HE-2026-0743, HE-2026-0744, HE-2026-0745, HE-2026-0746, HE-2026-0747, HE-2026-0748</t>
         </is>
       </c>
       <c r="R348" s="2" t="inlineStr"/>
@@ -45400,7 +45416,11 @@
           <t>1VdPtNYFiYsphBRUvCKB5muOHPFbq4537pancQrtGNiQ</t>
         </is>
       </c>
-      <c r="Q735" s="2" t="inlineStr"/>
+      <c r="Q735" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre en el formato actual (Mónica).</t>
+        </is>
+      </c>
       <c r="R735" s="2" t="inlineStr"/>
       <c r="S735" s="4" t="inlineStr"/>
     </row>
@@ -45459,7 +45479,7 @@
       </c>
       <c r="Q736" s="2" t="inlineStr">
         <is>
-          <t>aparte de sus versiones (leído): Las dos de 25-abr son el mismo Google Doc (mismo id) renombrado, proyecto de ascensor más subvenciones; la de 18-sep queda aparte porque solo trae subvenciones con IEE/CEE, sin proyecto, y no se sabe si sustituye a la de abril o es un encargo nuevo.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre en el formato actual (Mónica).</t>
         </is>
       </c>
       <c r="R736" s="2" t="inlineStr"/>
@@ -45689,7 +45709,11 @@
           <t>1sHssC7rfrJzaZZDNikOfZ8rDtRmjShctTDBlh9exJjA</t>
         </is>
       </c>
-      <c r="Q740" s="2" t="inlineStr"/>
+      <c r="Q740" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): En enero pidieron precio y se mandó todo junto; en septiembre retomaron y pidieron las hojas renovadas (Mónica).</t>
+        </is>
+      </c>
       <c r="R740" s="2" t="inlineStr"/>
       <c r="S740" s="4" t="inlineStr"/>
     </row>
@@ -45748,7 +45772,7 @@
       </c>
       <c r="Q741" s="2" t="inlineStr">
         <is>
-          <t>PARA TI · ¿versión o distinta?: La de enero es proyecto de ascensor (7.500) + subvención accesibilidad (1.980 fijo); la de septiembre es solo subvenciones accesibilidad a éxito (3,5%) + documentación técnica 1.980, sin proyecto: no se sabe si sustituye a la de enero (la comunidad renunció al proyecto) o es un encargo nuevo de subvención; ninguna firmada.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): En enero pidieron precio y se mandó todo junto; en septiembre retomaron y pidieron las hojas renovadas (Mónica).</t>
         </is>
       </c>
       <c r="R741" s="2" t="inlineStr"/>
@@ -45921,7 +45945,11 @@
           <t>13QCKnA2Jng553Spp341X9Hknf3lRQKuoD2xY9LFJ3Ho</t>
         </is>
       </c>
-      <c r="Q744" s="2" t="inlineStr"/>
+      <c r="Q744" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
+        </is>
+      </c>
       <c r="R744" s="2" t="inlineStr"/>
       <c r="S744" s="4" t="inlineStr"/>
     </row>
@@ -45978,7 +46006,11 @@
           <t>1wRjMx6loBIW14ZUg26kn1oWRQeIgc-OYjWYpWv3j5eU</t>
         </is>
       </c>
-      <c r="Q745" s="2" t="inlineStr"/>
+      <c r="Q745" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
+        </is>
+      </c>
       <c r="R745" s="2" t="inlineStr"/>
       <c r="S745" s="4" t="inlineStr"/>
     </row>
@@ -46035,7 +46067,11 @@
           <t>13QCKnA2Jng553Spp341X9Hknf3lRQKuoD2xY9LFJ3Ho</t>
         </is>
       </c>
-      <c r="Q746" s="2" t="inlineStr"/>
+      <c r="Q746" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
+        </is>
+      </c>
       <c r="R746" s="2" t="inlineStr"/>
       <c r="S746" s="4" t="inlineStr"/>
     </row>
@@ -46094,7 +46130,7 @@
       </c>
       <c r="Q747" s="2" t="inlineStr">
         <is>
-          <t>PARA TI · ¿versión o distinta?: La del 05-05 es proyecto de ascensor + subvenciones (nº 2026/04/056); las dos del 25-09 son solo subvenciones a éxito + doc. técnica 1.980, una de accesibilidad y otra de accesibilidad + eficiencia energética (más libro del edificio), con la misma fecha: parecen alternativas enviadas a la vez y no se sabe si sustituyen a la de mayo o son un encargo nuevo de subvención.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
         </is>
       </c>
       <c r="R747" s="2" t="inlineStr"/>
@@ -46155,7 +46191,7 @@
       </c>
       <c r="Q748" s="2" t="inlineStr">
         <is>
-          <t>PARA TI · ¿versión o distinta?: La del 05-05 es proyecto de ascensor + subvenciones (nº 2026/04/056); las dos del 25-09 son solo subvenciones a éxito + doc. técnica 1.980, una de accesibilidad y otra de accesibilidad + eficiencia energética (más libro del edificio), con la misma fecha: parecen alternativas enviadas a la vez y no se sabe si sustituyen a la de mayo o son un encargo nuevo de subvención.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
         </is>
       </c>
       <c r="R748" s="2" t="inlineStr"/>
@@ -46214,7 +46250,11 @@
           <t>1lz4SuZo3JwzjbkuCrVum1wcGoG_IazvHq9eajoQhTPo</t>
         </is>
       </c>
-      <c r="Q749" s="2" t="inlineStr"/>
+      <c r="Q749" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo caso: renovadas en septiembre, con alternativas (ascensor, SATE o conjunto; y sus subvenciones) (Mónica).</t>
+        </is>
+      </c>
       <c r="R749" s="2" t="inlineStr"/>
       <c r="S749" s="4" t="inlineStr"/>
     </row>
@@ -46271,7 +46311,11 @@
           <t>1xpmoBr9ktq3cCr_o4dswH6CZ3b62DsStDQ3hAJ2D4Dg</t>
         </is>
       </c>
-      <c r="Q750" s="2" t="inlineStr"/>
+      <c r="Q750" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo patrón y mismo administrador que Joaquina Santander 37 (aplicado por analogía; confirmar).</t>
+        </is>
+      </c>
       <c r="R750" s="2" t="inlineStr"/>
       <c r="S750" s="4" t="inlineStr"/>
     </row>
@@ -46328,7 +46372,11 @@
           <t>1kIDTFMCnhkpG3-TbFoMAhCwASmpGavSRGRnOuwVn6A8</t>
         </is>
       </c>
-      <c r="Q751" s="2" t="inlineStr"/>
+      <c r="Q751" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Mismo patrón y mismo administrador que Joaquina Santander 37 (aplicado por analogía; confirmar).</t>
+        </is>
+      </c>
       <c r="R751" s="2" t="inlineStr"/>
       <c r="S751" s="4" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Manifiesto 2026: sustituidas leidas e id de Drive por el titulo exacto
El id se adivinaba por fecha y direccion y fallaba cuando ese dia habia
varias hojas de la misma direccion. Ahora sale del listado de la carpeta
en Drive (drive_automaticas.tsv) por el titulo exacto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/manifiesto_hojas_2026.xlsx
+++ b/docs/manifiesto_hojas_2026.xlsx
@@ -1350,21 +1350,9 @@
           <t>2026-01-13</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>SAN HERCULANO 2 MADRID</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>ENVOLVENTE TERMICA</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, SATE CON CESION DE CAES</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1377,14 +1365,10 @@
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>1IA7ynbOYHlAkgHxEeteinTRX_fqTZ4Y5hw7RxQn4lCA</t>
+          <t>1tAggGlXVG54YqnkLGwWoFUMrxetBLlbdYv8haCXrNHk</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
@@ -1397,9 +1381,9 @@
           <t>HE-2026-0014</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1444,7 +1428,12 @@
           <t>1hzLLXH9kWAkW5ZHy_WJMLtg7YMcmC1cy9aDLdEN4arw</t>
         </is>
       </c>
-      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La de enero (envolvente/SATE + subvención eficiencia energética + CAES, 8.500 €) se reofertó en julio partida en proyecto SATE+CSS y tramitación de subvenciones de eficiencia; el elevador con derribo y la subvención de accesibilidad de septiembre son otro encargo.
+sustituida por: HE-2026-0639, HE-2026-0640</t>
+        </is>
+      </c>
       <c r="R15" s="2" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr"/>
     </row>
@@ -1946,12 +1935,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t xml:space="preserve">ACCESIBILIDAD </t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -2000,7 +1989,7 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>1phZvPmxJOGDf4dpHQRyGT7rxGGrpK0M3l4HMGKdmKzg</t>
+          <t>1sbpGkLc0TCcH6WFxgsq4Xgtq99Ims2_dIY2Qadhj6YU</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr"/>
@@ -2576,12 +2565,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -2603,7 +2592,7 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>1vwmQIhMx3w319k9GiQEdvvTR8HqY8MwYdKG2NuowPKU</t>
+          <t>10IDIMVeAhubxDBpdmetYyKAHn5uRuYm5FQe0SnHnFmI</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
@@ -4986,9 +4975,9 @@
           <t>HE-2026-0069</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5033,7 +5022,12 @@
           <t>1wxQ_C55MSIrc7uUnIbMT4zlPWIOPb_CB8lDSzSgS38o</t>
         </is>
       </c>
-      <c r="Q70" s="2" t="inlineStr"/>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) El propio título dice 'NO VALE, SE REOFERTÓ'; mismo proyecto SATE + subvención, reofertado rectificado en febrero (id real 1nkcGq7t...).
+sustituida por: HE-2026-0177</t>
+        </is>
+      </c>
       <c r="R70" s="2" t="inlineStr"/>
       <c r="S70" s="4" t="inlineStr"/>
     </row>
@@ -5575,9 +5569,21 @@
           <t>2026-02-03</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr"/>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>RONDA DE TOLEDO 40 MADRID</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>ACCESIBILIDAD CON PLATAFORMA ELEVADORA</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -5590,8 +5596,16 @@
       <c r="L79" s="2" t="n"/>
       <c r="M79" s="2" t="n"/>
       <c r="N79" s="2" t="n"/>
-      <c r="O79" s="2" t="n"/>
-      <c r="P79" s="2" t="n"/>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>1jg9PsJvyw9eabRJSpZwRWOF1SEw_CmN56VQwATzblZ4</t>
+        </is>
+      </c>
       <c r="Q79" s="2" t="inlineStr"/>
       <c r="R79" s="2" t="inlineStr"/>
       <c r="S79" s="4" t="inlineStr"/>
@@ -6742,21 +6756,9 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>NURIA 28-32 MADRID</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>ACCESIBILIDAD</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -6769,14 +6771,10 @@
       <c r="L95" s="2" t="n"/>
       <c r="M95" s="2" t="n"/>
       <c r="N95" s="2" t="n"/>
-      <c r="O95" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="O95" s="2" t="n"/>
       <c r="P95" s="2" t="inlineStr">
         <is>
-          <t>1OcxatE-zjorsicjX9s5apUC8CLv-Quc9OFp_Zcn-y6s</t>
+          <t>1S0CGnusIOVQ7xxXYuxcFOWUP1X-xOIcoAh_C99EEmjI</t>
         </is>
       </c>
       <c r="Q95" s="2" t="inlineStr"/>
@@ -6891,12 +6889,12 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>ACCESIBILIDAD</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
@@ -6942,7 +6940,7 @@
       </c>
       <c r="P97" s="2" t="inlineStr">
         <is>
-          <t>1OcxatE-zjorsicjX9s5apUC8CLv-Quc9OFp_Zcn-y6s</t>
+          <t>1_NGscsM-zDKiaPFdxg2DDLAsVPfZkg8GH2U5FAntWI0</t>
         </is>
       </c>
       <c r="Q97" s="2" t="inlineStr"/>
@@ -7126,9 +7124,9 @@
           <t>HE-2026-0100</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -7173,7 +7171,12 @@
           <t>1yib07QXRtskyYqjTaxkhXJWnB_q_w8ZczuOvwN7yb7A</t>
         </is>
       </c>
-      <c r="Q101" s="2" t="inlineStr"/>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) El PRY ASCENSOR + SUBV de febrero se reofertó en mayo partido en proyecto ascensor y tramitación de subvenciones con IEE/CEE (formato actual).
+sustituida por: HE-2026-0458, HE-2026-0459</t>
+        </is>
+      </c>
       <c r="R101" s="2" t="inlineStr"/>
       <c r="S101" s="4" t="inlineStr"/>
     </row>
@@ -7200,12 +7203,12 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr"/>
@@ -7227,7 +7230,7 @@
       </c>
       <c r="P102" s="2" t="inlineStr">
         <is>
-          <t>1yib07QXRtskyYqjTaxkhXJWnB_q_w8ZczuOvwN7yb7A</t>
+          <t>1-vlVkIfXH9DDE2bTenhyiNN3DU5KpiXl5ccy9yJlewU</t>
         </is>
       </c>
       <c r="Q102" s="2" t="inlineStr"/>
@@ -7240,9 +7243,9 @@
           <t>HE-2026-0102</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -7266,8 +7269,17 @@
       <c r="M103" s="2" t="n"/>
       <c r="N103" s="2" t="n"/>
       <c r="O103" s="2" t="n"/>
-      <c r="P103" s="2" t="n"/>
-      <c r="Q103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>1s7fIZ0p8kdqg_MTB5r2E0MzuPUw_2C5yuGACips5pD0</t>
+        </is>
+      </c>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) El proyecto de ascensor + subvención accesibilidad de febrero se renovó en mayo partido en proyecto de ascensor (+CSS) y tramitación de subvenciones con el formato actual.
+sustituida por: HE-2026-0460, HE-2026-0461</t>
+        </is>
+      </c>
       <c r="R103" s="2" t="inlineStr"/>
       <c r="S103" s="4" t="inlineStr"/>
     </row>
@@ -7303,7 +7315,11 @@
       <c r="M104" s="2" t="n"/>
       <c r="N104" s="2" t="n"/>
       <c r="O104" s="2" t="n"/>
-      <c r="P104" s="2" t="n"/>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>1TkgvPFZlTdO72Ciih7hL__3D2l-pXvRAcanPY3pAkQg</t>
+        </is>
+      </c>
       <c r="Q104" s="2" t="inlineStr"/>
       <c r="R104" s="2" t="inlineStr"/>
       <c r="S104" s="4" t="inlineStr"/>
@@ -7340,7 +7356,11 @@
       <c r="M105" s="2" t="n"/>
       <c r="N105" s="2" t="n"/>
       <c r="O105" s="2" t="n"/>
-      <c r="P105" s="2" t="n"/>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>1Izxw6O8lR9nSuwDQQuOvF8d-L4R_4aUGf2MfniVvcKs</t>
+        </is>
+      </c>
       <c r="Q105" s="2" t="inlineStr"/>
       <c r="R105" s="2" t="inlineStr"/>
       <c r="S105" s="4" t="inlineStr"/>
@@ -7377,7 +7397,11 @@
       <c r="M106" s="2" t="n"/>
       <c r="N106" s="2" t="n"/>
       <c r="O106" s="2" t="n"/>
-      <c r="P106" s="2" t="n"/>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>11ZP2CCY8SwX4mXCcFZw8bgwJBNk2_Bo7OmttRUlTpUY</t>
+        </is>
+      </c>
       <c r="Q106" s="2" t="inlineStr"/>
       <c r="R106" s="2" t="inlineStr"/>
       <c r="S106" s="4" t="inlineStr"/>
@@ -7405,12 +7429,12 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr"/>
@@ -7432,7 +7456,7 @@
       </c>
       <c r="P107" s="2" t="inlineStr">
         <is>
-          <t>1ddRCF3wRw6LJSGRUbmz4minF_TRAj9aGWmKw_DmcwiE</t>
+          <t>1_v3eRPWTDKWAzHAex1GOtqNsSTa9cih8ehhqpDPZXIg</t>
         </is>
       </c>
       <c r="Q107" s="2" t="inlineStr"/>
@@ -7756,12 +7780,12 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
@@ -7783,7 +7807,7 @@
       </c>
       <c r="P112" s="2" t="inlineStr">
         <is>
-          <t>1SnopyhtMq-AG6j2pWTYfPCOEPeyrWvpP8cFlhYjhkG8</t>
+          <t>1nhv-7_cdwvFQFulb9-yuEAPboFAU7ahqSxIul5aEZT8</t>
         </is>
       </c>
       <c r="Q112" s="2" t="inlineStr"/>
@@ -7813,12 +7837,12 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, SATE CON CESION DE CAES</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr"/>
@@ -7840,7 +7864,7 @@
       </c>
       <c r="P113" s="2" t="inlineStr">
         <is>
-          <t>1SnopyhtMq-AG6j2pWTYfPCOEPeyrWvpP8cFlhYjhkG8</t>
+          <t>1XE5dIeFBbN-2uLPhdZtujM7URNd0yeNdPMuyzEpWuPU</t>
         </is>
       </c>
       <c r="Q113" s="2" t="inlineStr"/>
@@ -7927,12 +7951,12 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA</t>
+          <t>INSTALACIÓN DE ASCENSOR</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE, SATE CON CESION DE CAES</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
@@ -7982,7 +8006,7 @@
       </c>
       <c r="P115" s="2" t="inlineStr">
         <is>
-          <t>1SLfiAtqtS61i2AyzfagwhamKeGz135oUeSynfMi3_xo</t>
+          <t>1dOp9hDuXEC3mz9-n7THvj-FwwSCxpmYPl-qvVw1UdxU</t>
         </is>
       </c>
       <c r="Q115" s="2" t="inlineStr"/>
@@ -8044,7 +8068,8 @@
       </c>
       <c r="Q116" s="2" t="inlineStr">
         <is>
-          <t>hoja distinta, no versión (leído): Objetos distintos: la del 10-02 es proyecto de envolvente térmica (SATE con cesión de CAES, 18.220) y la del 16-02 es proyecto de cubierta (7.000); la firmada es la de cubierta.</t>
+          <t>hoja distinta, no versión (leído): Objetos distintos: la del 10-02 es proyecto de envolvente térmica (SATE con cesión de CAES, 18.220) y la del 16-02 es proyecto de cubierta (7.000); la firmada es la de cubierta.
+PARA TI · ¿sustituida por una posterior?: La antigua es proyecto SATE de fachada + subvención EE con CAES; las posteriores son proyecto de CUBIERTA y subvención de ACCESIBILIDAD (que casa con la hoja ASC2), ninguna recoge el SATE: puede que lo cambiaran por cubierta o que siga aparte.</t>
         </is>
       </c>
       <c r="R116" s="2" t="inlineStr"/>
@@ -9019,12 +9044,12 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>IEE</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>IEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE, SATE CON CESION DE CAES</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr"/>
@@ -9046,7 +9071,7 @@
       </c>
       <c r="P133" s="2" t="inlineStr">
         <is>
-          <t>10UzO5ky7IhJEfxvgrZb0HBkhMJyr9YQ-s6z6bl36LTA</t>
+          <t>1YaTr2vIjOSru8rMSlufGjjfpbDlYIZpT9I6NvtEc3LQ</t>
         </is>
       </c>
       <c r="Q133" s="2" t="inlineStr"/>
@@ -9529,8 +9554,16 @@
           <t>PEDRO UNANUME 22 MADRID</t>
         </is>
       </c>
-      <c r="E141" s="2" t="n"/>
-      <c r="F141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>INFORME PARA CONTESTACIÓN DE REQUERIMIENTO</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>INFORME PERICIAL</t>
+        </is>
+      </c>
       <c r="G141" s="2" t="inlineStr"/>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -9565,8 +9598,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O141" s="2" t="n"/>
-      <c r="P141" s="2" t="n"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>1lQzszHUcRErl1Xx0AXwqv8zh1RhGlzKJzgIpIvzprb4</t>
+        </is>
+      </c>
       <c r="Q141" s="2" t="inlineStr">
         <is>
           <t>tanda1 101: RESUELTO LEYENDO: La hoja dice 'UNANUME' (errata); la dirección buena es la de la opp.</t>
@@ -9721,7 +9762,11 @@
       <c r="M144" s="2" t="n"/>
       <c r="N144" s="2" t="n"/>
       <c r="O144" s="2" t="n"/>
-      <c r="P144" s="2" t="n"/>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>15kTuFcaLkU8L30rIezzbEhOTKdU9Snl124SO7vsutaQ</t>
+        </is>
+      </c>
       <c r="Q144" s="2" t="inlineStr"/>
       <c r="R144" s="2" t="inlineStr"/>
       <c r="S144" s="4" t="inlineStr"/>
@@ -10151,16 +10196,8 @@
           <t>AV DOCTOR GARCIA TAPIA NUM 133-135-137 MADRID</t>
         </is>
       </c>
-      <c r="E151" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DF Y CERTIFICADO DE IDONIEDAD </t>
-        </is>
-      </c>
-      <c r="F151" s="2" t="inlineStr">
-        <is>
-          <t>DF, INFORME PERICIAL</t>
-        </is>
-      </c>
+      <c r="E151" s="2" t="n"/>
+      <c r="F151" s="2" t="inlineStr"/>
       <c r="G151" s="2" t="inlineStr"/>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -10196,14 +10233,10 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O151" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O151" s="2" t="n"/>
       <c r="P151" s="2" t="inlineStr">
         <is>
-          <t>1_iDFiPzplECsmCrgqlw_RFwOJGo2j6zCbBLZaPNuP1Y</t>
+          <t>1VDqkv9TE6uCVIVk_ZlSTMCdz7SQEg79CzgHkEmW6DPI</t>
         </is>
       </c>
       <c r="Q151" s="2" t="inlineStr"/>
@@ -10994,21 +11027,9 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t>ARROYO MEDIA LEGUA 30 MADRID</t>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ASCENSOR Y ENVOLVENTE TERMICA </t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
-        </is>
-      </c>
+      <c r="D165" s="2" t="inlineStr"/>
+      <c r="E165" s="2" t="n"/>
+      <c r="F165" s="2" t="inlineStr"/>
       <c r="G165" s="2" t="inlineStr"/>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -11021,14 +11042,10 @@
       <c r="L165" s="2" t="n"/>
       <c r="M165" s="2" t="n"/>
       <c r="N165" s="2" t="n"/>
-      <c r="O165" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O165" s="2" t="n"/>
       <c r="P165" s="2" t="inlineStr">
         <is>
-          <t>1fRaBVVyvBNeuIQOfInlDGWGqmGs0iAHpjbZkDCY9TMw</t>
+          <t>1D0Gx95VpCcxctdlUJbzd6eLkZeDDyzWPS7c27rA7e4w</t>
         </is>
       </c>
       <c r="Q165" s="2" t="inlineStr"/>
@@ -11067,7 +11084,11 @@
       <c r="M166" s="2" t="n"/>
       <c r="N166" s="2" t="n"/>
       <c r="O166" s="2" t="n"/>
-      <c r="P166" s="2" t="n"/>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>1HXxlp6te7Ca7yzIiAlmX6PxBMuNd3ykkkpREJc39bNQ</t>
+        </is>
+      </c>
       <c r="Q166" s="2" t="inlineStr"/>
       <c r="R166" s="2" t="inlineStr"/>
       <c r="S166" s="4" t="inlineStr"/>
@@ -11104,7 +11125,11 @@
       <c r="M167" s="2" t="n"/>
       <c r="N167" s="2" t="n"/>
       <c r="O167" s="2" t="n"/>
-      <c r="P167" s="2" t="n"/>
+      <c r="P167" s="2" t="inlineStr">
+        <is>
+          <t>1L2c5Zxptzlef8YvmnA3u_ac9MX8FyIL4PaBZfIJwAn4</t>
+        </is>
+      </c>
       <c r="Q167" s="2" t="inlineStr"/>
       <c r="R167" s="2" t="inlineStr"/>
       <c r="S167" s="4" t="inlineStr"/>
@@ -11130,8 +11155,16 @@
           <t>CASIMIRO ESCUDERO 11 MADRID</t>
         </is>
       </c>
-      <c r="E168" s="2" t="n"/>
-      <c r="F168" s="2" t="inlineStr"/>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>IEE</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>IEE</t>
+        </is>
+      </c>
       <c r="G168" s="2" t="inlineStr"/>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -11166,8 +11199,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O168" s="2" t="n"/>
-      <c r="P168" s="2" t="n"/>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>1WvAlK_oCOlfzqluC5esGHenjKr9_kDzdEJiVRe95FPo</t>
+        </is>
+      </c>
       <c r="Q168" s="2" t="inlineStr"/>
       <c r="R168" s="2" t="inlineStr"/>
       <c r="S168" s="4" t="inlineStr"/>
@@ -11193,16 +11234,8 @@
           <t>CASTELLON 15 MOSTOLES</t>
         </is>
       </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>ENVOLVENTE TERMICA</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
-        </is>
-      </c>
+      <c r="E169" s="2" t="n"/>
+      <c r="F169" s="2" t="inlineStr"/>
       <c r="G169" s="2" t="inlineStr">
         <is>
           <t>v1 2026-02-25 · CASTELLON 15 MOSTOLES - 25 02 2026 - PRY SATE+SUBV.gdoc  ← FIRMADA
@@ -11252,14 +11285,10 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O169" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O169" s="2" t="n"/>
       <c r="P169" s="2" t="inlineStr">
         <is>
-          <t>1uGjv2l0dH8NAxOceBJLUiOdDkFTe5wZqD8LKvCF87WA</t>
+          <t>1v0MLvq5bIT72HX-wqqMg4ppI6aCr-IHTxfPqN0xu1wY</t>
         </is>
       </c>
       <c r="Q169" s="2" t="inlineStr">
@@ -11437,16 +11466,8 @@
           <t>ISAAC PERAL 5 MOSTOLES</t>
         </is>
       </c>
-      <c r="E172" s="2" t="inlineStr">
-        <is>
-          <t>ENVOLVENTE TERMICA</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
-        </is>
-      </c>
+      <c r="E172" s="2" t="n"/>
+      <c r="F172" s="2" t="inlineStr"/>
       <c r="G172" s="2" t="inlineStr">
         <is>
           <t>v1 2026-02-25 · ISAAC PERAL 5 MOSTOLES - 25 02 2026 - PRY SATE+SUBV.gdoc  ← FIRMADA
@@ -11496,14 +11517,10 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O172" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O172" s="2" t="n"/>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>1FkCiyidfBVl-_g9JG-ZQs1_bpSpHIK1tvdxy0D5eEdo</t>
+          <t>18pIf0QQst3EWssKYG4UqDzcKRFbIbLB8FXWGhPpbaSo</t>
         </is>
       </c>
       <c r="Q172" s="2" t="inlineStr">
@@ -11891,16 +11908,8 @@
           <t>SIMON HERNANDEZ 43-45 MOSTOLES</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
-        <is>
-          <t>ENVOLVENTE TERMICA</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
-        </is>
-      </c>
+      <c r="E177" s="2" t="n"/>
+      <c r="F177" s="2" t="inlineStr"/>
       <c r="G177" s="2" t="inlineStr">
         <is>
           <t>v1 2026-02-25 · SIMON HERNANDEZ 43-45 MOSTOLES - 25 02 2026 - PRY SATE+SUBV.gdoc
@@ -11950,14 +11959,10 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O177" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O177" s="2" t="n"/>
       <c r="P177" s="2" t="inlineStr">
         <is>
-          <t>1Lyn44toYFhAijvCIUZUdPTge6N7d1may0kJ5Gu_q47M</t>
+          <t>1ZSYC77NSp6fUK7uygg5zyrlXfGP9nZRkBcmvLA4vyvI</t>
         </is>
       </c>
       <c r="Q177" s="2" t="inlineStr">
@@ -11984,9 +11989,21 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr"/>
-      <c r="E178" s="2" t="n"/>
-      <c r="F178" s="2" t="inlineStr"/>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>SIMON HERNANDEZ 42 MOSTOLES</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>ENVOLVENTE TERMICA</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+        </is>
+      </c>
       <c r="G178" s="2" t="inlineStr"/>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -11999,9 +12016,21 @@
       <c r="L178" s="2" t="n"/>
       <c r="M178" s="2" t="n"/>
       <c r="N178" s="2" t="n"/>
-      <c r="O178" s="2" t="n"/>
-      <c r="P178" s="2" t="n"/>
-      <c r="Q178" s="2" t="inlineStr"/>
+      <c r="O178" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P178" s="2" t="inlineStr">
+        <is>
+          <t>1nkcGq7t_nT0hK3g46ztow9GkDkZA_Pfg2S9YOwv7R9o</t>
+        </is>
+      </c>
+      <c r="Q178" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El propio título dice 'NO VALE, SE REOFERTÓ'; mismo proyecto SATE + subvención, reofertado rectificado en febrero (id real 1nkcGq7t...).</t>
+        </is>
+      </c>
       <c r="R178" s="2" t="inlineStr"/>
       <c r="S178" s="4" t="inlineStr"/>
     </row>
@@ -12271,9 +12300,21 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr"/>
-      <c r="E183" s="2" t="n"/>
-      <c r="F183" s="2" t="inlineStr"/>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>BLAS CABRERA 44 MADRID</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACIÓN DE ASCENSOR</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+        </is>
+      </c>
       <c r="G183" s="2" t="inlineStr"/>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -12286,8 +12327,16 @@
       <c r="L183" s="2" t="n"/>
       <c r="M183" s="2" t="n"/>
       <c r="N183" s="2" t="n"/>
-      <c r="O183" s="2" t="n"/>
-      <c r="P183" s="2" t="n"/>
+      <c r="O183" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P183" s="2" t="inlineStr">
+        <is>
+          <t>16QzIRc0CfX9AY9DTCCmHRKzU53VmRR0fadq0z41ojfs</t>
+        </is>
+      </c>
       <c r="Q183" s="2" t="inlineStr"/>
       <c r="R183" s="2" t="inlineStr"/>
       <c r="S183" s="4" t="inlineStr"/>
@@ -12657,12 +12706,12 @@
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ASCENSOR</t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+          <t>REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -12685,12 +12734,12 @@
       <c r="N190" s="2" t="n"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>1cbCMhMfShOUCvnIuD9VLfgDan_GV3ljgkU0TSbk2x9M</t>
+          <t>1NDv7FANukiIm3Sq-Qb9iHq89IMoeTKCk6DCZWHTOzgo</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr"/>
@@ -13408,21 +13457,9 @@
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
-        <is>
-          <t>FELIPE DIAZ 3 MADRID</t>
-        </is>
-      </c>
-      <c r="E202" s="2" t="inlineStr">
-        <is>
-          <t>ENVOLVENTE TERMICA</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, CEE, SATE CON CESION DE CAES</t>
-        </is>
-      </c>
+      <c r="D202" s="2" t="inlineStr"/>
+      <c r="E202" s="2" t="n"/>
+      <c r="F202" s="2" t="inlineStr"/>
       <c r="G202" s="2" t="inlineStr"/>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -13435,14 +13472,10 @@
       <c r="L202" s="2" t="n"/>
       <c r="M202" s="2" t="n"/>
       <c r="N202" s="2" t="n"/>
-      <c r="O202" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="O202" s="2" t="n"/>
       <c r="P202" s="2" t="inlineStr">
         <is>
-          <t>1JgfxDXvsWtZtVoIhzqa-VnG97o5NiX6VTSZoZVaIEKk</t>
+          <t>17kfVzx5ufod8E_aotUcYd7Hu3DPjtfO04Dcu6GQq4B0</t>
         </is>
       </c>
       <c r="Q202" s="2" t="inlineStr"/>
@@ -13527,8 +13560,16 @@
           <t>LAS PALMAS 43 MÓSTOLES</t>
         </is>
       </c>
-      <c r="E204" s="2" t="n"/>
-      <c r="F204" s="2" t="inlineStr"/>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>ACCESIBILIDAD</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G204" s="2" t="inlineStr"/>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -13564,8 +13605,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O204" s="2" t="n"/>
-      <c r="P204" s="2" t="n"/>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr">
+        <is>
+          <t>1t2Lh8dd75spE5NuvOAXUKf8ImH7wvafYrMq3b2lxiII</t>
+        </is>
+      </c>
       <c r="Q204" s="2" t="inlineStr"/>
       <c r="R204" s="2" t="inlineStr"/>
       <c r="S204" s="4" t="inlineStr"/>
@@ -14220,12 +14269,12 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>MODIFICACION DE ASCENSOR</t>
+          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr"/>
@@ -14247,7 +14296,7 @@
       </c>
       <c r="P216" s="2" t="inlineStr">
         <is>
-          <t>1nQyjXcfktWO6BTbilpW411zVNgY2gljhb4qXOagHEJA</t>
+          <t>1NYGNTJVkebvTLADZql-aeF8-c6YbiJ2wLqSaA5U-p-Y</t>
         </is>
       </c>
       <c r="Q216" s="2" t="inlineStr"/>
@@ -14686,9 +14735,9 @@
           <t>HE-2026-0223</t>
         </is>
       </c>
-      <c r="B224" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B224" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
@@ -14733,7 +14782,12 @@
           <t>1TpQMwOB5c-_Eb4iOuPOzmwp9JZgjon3dLmugQuC8ifE</t>
         </is>
       </c>
-      <c r="Q224" s="2" t="inlineStr"/>
+      <c r="Q224" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Misma CSS de 920 € para la misma obra, reemitida con formato actual y numeración; la posterior se firmó.
+sustituida por: HE-2026-0272</t>
+        </is>
+      </c>
       <c r="R224" s="2" t="inlineStr"/>
       <c r="S224" s="4" t="inlineStr"/>
     </row>
@@ -14800,9 +14854,9 @@
           <t>HE-2026-0225</t>
         </is>
       </c>
-      <c r="B226" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B226" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
@@ -14847,7 +14901,12 @@
           <t>1WY92Sje8aYpmF-uSzCrzTI77Vqwt1em_8sUbBb4-tRY</t>
         </is>
       </c>
-      <c r="Q226" s="2" t="inlineStr"/>
+      <c r="Q226" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Proyecto de ascensor + subvención accesibilidad de marzo renovado en julio separado en proyecto de ascensor (+CSS, pago fraccionado) y tramitación de subvenciones de accesibilidad.
+sustituida por: HE-2026-0621, HE-2026-0622</t>
+        </is>
+      </c>
       <c r="R226" s="2" t="inlineStr"/>
       <c r="S226" s="4" t="inlineStr"/>
     </row>
@@ -16861,7 +16920,7 @@
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AISLAMIENTO DE CUBIERTA </t>
+          <t>CUBIERTA Y FACHADA (SATE)</t>
         </is>
       </c>
       <c r="F259" s="2" t="inlineStr">
@@ -16888,7 +16947,7 @@
       </c>
       <c r="P259" s="2" t="inlineStr">
         <is>
-          <t>1iHFIrEfy1HXRmx-xBmuybdoF_VDUaxbc8R0YQzahZiU</t>
+          <t>1meqOubVJG2P_gMCUlu9cPYboJE56McNBKILUgkzVhPM</t>
         </is>
       </c>
       <c r="Q259" s="2" t="inlineStr"/>
@@ -17109,9 +17168,21 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="D263" s="2" t="inlineStr"/>
-      <c r="E263" s="2" t="n"/>
-      <c r="F263" s="2" t="inlineStr"/>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>PIQUEÑAS 14 MADRID</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACIÓN ASCENSOR</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+        </is>
+      </c>
       <c r="G263" s="2" t="inlineStr"/>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -17124,8 +17195,16 @@
       <c r="L263" s="2" t="n"/>
       <c r="M263" s="2" t="n"/>
       <c r="N263" s="2" t="n"/>
-      <c r="O263" s="2" t="n"/>
-      <c r="P263" s="2" t="n"/>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="inlineStr">
+        <is>
+          <t>1AVFmxTT6AXGQQRTwfjuQoP9LiO7rnq3BpMPK283rYv4</t>
+        </is>
+      </c>
       <c r="Q263" s="2" t="inlineStr"/>
       <c r="R263" s="2" t="inlineStr"/>
       <c r="S263" s="4" t="inlineStr"/>
@@ -17153,12 +17232,12 @@
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SATE </t>
+          <t>SUBSANACIÓN IEE</t>
         </is>
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr"/>
@@ -17180,7 +17259,7 @@
       </c>
       <c r="P264" s="2" t="inlineStr">
         <is>
-          <t>1ViVr_lSvu0HvMcTFgFxWzm4ik3yZieYToS_B5HW43dI</t>
+          <t>1BlpTjUxpCublBT_n32rBlKAnh7yhv4ZpZTeMQ5ePf08</t>
         </is>
       </c>
       <c r="Q264" s="2" t="inlineStr"/>
@@ -17193,9 +17272,9 @@
           <t>HE-2026-0264</t>
         </is>
       </c>
-      <c r="B265" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B265" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
@@ -17240,7 +17319,12 @@
           <t>1ViVr_lSvu0HvMcTFgFxWzm4ik3yZieYToS_B5HW43dI</t>
         </is>
       </c>
-      <c r="Q265" s="2" t="inlineStr"/>
+      <c r="Q265" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Mismo proyecto SATE (mismo PEM 490.000/550.000 €) reofertado con formato actual, honorarios 24.010 € y subvención solo a éxito.
+sustituida por: HE-2026-0368</t>
+        </is>
+      </c>
       <c r="R265" s="2" t="inlineStr"/>
       <c r="S265" s="4" t="inlineStr"/>
     </row>
@@ -17267,12 +17351,12 @@
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, LEE, CEE, SATE CON CESION DE CAES</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
@@ -17294,7 +17378,7 @@
       </c>
       <c r="P266" s="2" t="inlineStr">
         <is>
-          <t>1AVFmxTT6AXGQQRTwfjuQoP9LiO7rnq3BpMPK283rYv4</t>
+          <t>1hURUCQNBAd08V9dPIONpIm8Z_0IIoenXyDe6WZGSzho</t>
         </is>
       </c>
       <c r="Q266" s="2" t="inlineStr"/>
@@ -17766,7 +17850,11 @@
           <t>1w6uOl3B_0dxut5IYyGWIEl4m6sM2Ivq4emhJNaA6VVk</t>
         </is>
       </c>
-      <c r="Q273" s="2" t="inlineStr"/>
+      <c r="Q273" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Misma CSS de 920 € para la misma obra, reemitida con formato actual y numeración; la posterior se firmó.</t>
+        </is>
+      </c>
       <c r="R273" s="2" t="inlineStr"/>
       <c r="S273" s="4" t="inlineStr"/>
     </row>
@@ -18793,12 +18881,12 @@
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
+          <t>BAJADA A COTA 0</t>
         </is>
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr"/>
@@ -18820,7 +18908,7 @@
       </c>
       <c r="P290" s="2" t="inlineStr">
         <is>
-          <t>1bw-GJx3wYQxB4UUHP6XBB969F_QYU-cnRlpLPzQJzK0</t>
+          <t>1F_bmh3FQAmh8bwI3WdXTMW0Sir3lvc2V6Bjo0TYXi8k</t>
         </is>
       </c>
       <c r="Q290" s="2" t="inlineStr"/>
@@ -18890,9 +18978,9 @@
           <t>HE-2026-0291</t>
         </is>
       </c>
-      <c r="B292" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B292" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
@@ -18937,7 +19025,12 @@
           <t>14ZnAGulPyc9r6cHocf0hSe-bqDi_rgBrSXxDvEwPWuY</t>
         </is>
       </c>
-      <c r="Q292" s="2" t="inlineStr"/>
+      <c r="Q292" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La tramitación de subvenciones de accesibilidad del portal 1 (765 € fijo) se reofertó a los portales 1-2-3 juntos en junio, hoja firmada.
+sustituida por: HE-2026-0572</t>
+        </is>
+      </c>
       <c r="R292" s="2" t="inlineStr"/>
       <c r="S292" s="4" t="inlineStr"/>
     </row>
@@ -18947,9 +19040,9 @@
           <t>HE-2026-0292</t>
         </is>
       </c>
-      <c r="B293" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B293" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
@@ -18959,7 +19052,7 @@
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>NECTAR 31 PORTAL 1</t>
+          <t>NECTAR 31 PORTAL 1,2 Y 3</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -18991,10 +19084,15 @@
       </c>
       <c r="P293" s="2" t="inlineStr">
         <is>
-          <t>14ZnAGulPyc9r6cHocf0hSe-bqDi_rgBrSXxDvEwPWuY</t>
-        </is>
-      </c>
-      <c r="Q293" s="2" t="inlineStr"/>
+          <t>1veK70YDDclIIb6LRsif3qn_QHkJgHV7NAUWDXe9uqG8</t>
+        </is>
+      </c>
+      <c r="Q293" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Misma tramitación de subvenciones de accesibilidad del portal 1, reofertada a los portales 1-2-3 con el formato actual (doc. técnica 2.625 + 3,5%).
+sustituida por: HE-2026-0572</t>
+        </is>
+      </c>
       <c r="R293" s="2" t="inlineStr"/>
       <c r="S293" s="4" t="inlineStr"/>
     </row>
@@ -19004,9 +19102,9 @@
           <t>HE-2026-0293</t>
         </is>
       </c>
-      <c r="B294" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B294" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
@@ -19016,7 +19114,7 @@
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>NECTAR 31 PORTAL 1</t>
+          <t>NECTAR 31 PORTAL 2</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
@@ -19048,10 +19146,15 @@
       </c>
       <c r="P294" s="2" t="inlineStr">
         <is>
-          <t>14ZnAGulPyc9r6cHocf0hSe-bqDi_rgBrSXxDvEwPWuY</t>
-        </is>
-      </c>
-      <c r="Q294" s="2" t="inlineStr"/>
+          <t>1jhgdllKbTddUI5utZwlHhhQb4aXouaCGi_hdBMuNnkk</t>
+        </is>
+      </c>
+      <c r="Q294" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La tramitación de subvenciones de accesibilidad del portal se reofertó para los portales 1-2-3 (mancomunidad) con IEE/CEE; la posterior se firmó.
+sustituida por: HE-2026-0572</t>
+        </is>
+      </c>
       <c r="R294" s="2" t="inlineStr"/>
       <c r="S294" s="4" t="inlineStr"/>
     </row>
@@ -19061,9 +19164,9 @@
           <t>HE-2026-0294</t>
         </is>
       </c>
-      <c r="B295" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B295" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
@@ -19073,7 +19176,7 @@
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>NECTAR 31 PORTAL 1</t>
+          <t>NECTAR 31 PORTAL3</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
@@ -19105,10 +19208,15 @@
       </c>
       <c r="P295" s="2" t="inlineStr">
         <is>
-          <t>14ZnAGulPyc9r6cHocf0hSe-bqDi_rgBrSXxDvEwPWuY</t>
-        </is>
-      </c>
-      <c r="Q295" s="2" t="inlineStr"/>
+          <t>12vQf_87zQRhQEhEI6CFotsaDdebqDutD6WuLZlC7jao</t>
+        </is>
+      </c>
+      <c r="Q295" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La tramitación de subvenciones de accesibilidad del portal 3 (765 € fijo) se reofertó a los portales 1-2-3 juntos en junio, hoja firmada.
+sustituida por: HE-2026-0572</t>
+        </is>
+      </c>
       <c r="R295" s="2" t="inlineStr"/>
       <c r="S295" s="4" t="inlineStr"/>
     </row>
@@ -19118,9 +19226,9 @@
           <t>HE-2026-0295</t>
         </is>
       </c>
-      <c r="B296" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B296" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
@@ -19174,7 +19282,8 @@
       <c r="Q296" s="2" t="inlineStr">
         <is>
           <t>versiones (leído): Mismo encargo de proyecto de ascensor con IEE y CEE; la de mayo pasa a 2 ascensores y reparte los mismos 9.200 € en proyecto (8.280) y coordinación de seguridad (920).
-versiones (leído): Mismo encargo de proyecto de ascensor con IEE y CEE; la de mayo pasa a 2 ascensores y reparte los mismos 9.200 € en proyecto (8.280) y coordinación de seguridad (920).</t>
+SUSTITUIDA: (leído) El proyecto de 2 ascensores (8.280, con IEE/CEE) se reofertó ampliado con envolvente (23.000) y el IEE/CEE pasó a la hoja de subvenciones.
+sustituida por: HE-2026-0428, HE-2026-0429</t>
         </is>
       </c>
       <c r="R296" s="2" t="inlineStr"/>
@@ -19186,9 +19295,9 @@
           <t>HE-2026-0296</t>
         </is>
       </c>
-      <c r="B297" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B297" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
@@ -19242,7 +19351,8 @@
       <c r="Q297" s="2" t="inlineStr">
         <is>
           <t>versiones (leído): Mismo proyecto de fachada SATE (la v2 lo titula envolvente térmica y describe el SATE); sube de 14.790 € a 16.180 € + CSS 920 € y la obra estimada de 317.640 € a 440.000 €.
-versiones (leído): Mismo proyecto de fachada SATE (la v2 lo titula envolvente térmica y describe el SATE); sube de 14.790 € a 16.180 € + CSS 920 € y la obra estimada de 317.640 € a 440.000 €.</t>
+SUSTITUIDA: (leído) El proyecto de envolvente térmica (con IEE/CEE/libro) se reofertó como proyecto 2 ascensores + envolvente y aparte subvenciones accesibilidad y EE con la documentación técnica; ambas firmadas.
+sustituida por: HE-2026-0428, HE-2026-0429</t>
         </is>
       </c>
       <c r="R297" s="2" t="inlineStr"/>
@@ -19254,9 +19364,9 @@
           <t>HE-2026-0297</t>
         </is>
       </c>
-      <c r="B298" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B298" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
@@ -19310,7 +19420,8 @@
       <c r="Q298" s="2" t="inlineStr">
         <is>
           <t>versiones (leído): Mismo encargo de tramitación de subvenciones; la del 13-05 (nº 2026/05/017) amplía a accesibilidad + eficiencia energética y cambia honorarios (documentación técnica 1.980 + 3,5% a éxito) frente a solo eficiencia energética con 1.980 fijo + 3,5% de la del 13-04.
-versiones (leído): Mismo encargo de tramitación de subvenciones; la del 13-05 (nº 2026/05/017) amplía a accesibilidad + eficiencia energética y cambia honorarios (documentación técnica 1.980 + 3,5% a éxito) frente a solo eficiencia energética con 1.980 fijo + 3,5% de la del 13-04.</t>
+SUSTITUIDA: (leído) La tramitación de subvenciones de accesibilidad y eficiencia del 13-may se rehízo el 22-may (mismo objeto, 1.980 € + 3% a éxito) y es la firmada; el proyecto de 2 ascensores y envolvente es encargo aparte.
+sustituida por: HE-2026-0429</t>
         </is>
       </c>
       <c r="R298" s="2" t="inlineStr"/>
@@ -19624,12 +19735,12 @@
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA</t>
         </is>
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, SATE CON CESION DE CAES</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr"/>
@@ -19651,7 +19762,7 @@
       </c>
       <c r="P304" s="2" t="inlineStr">
         <is>
-          <t>1X9_XRG7HJhUOX7lYfdcttLMA34il0tUr6MrHv-oMaVQ</t>
+          <t>12Bkmugdd8BHn2I2P2HzLwlDvxks33KhQ_LbifSHABRc</t>
         </is>
       </c>
       <c r="Q304" s="2" t="inlineStr"/>
@@ -20216,9 +20327,21 @@
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="D313" s="2" t="inlineStr"/>
-      <c r="E313" s="2" t="n"/>
-      <c r="F313" s="2" t="inlineStr"/>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>VALDECANILLAS 82 MADRID</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>TRASTEROS</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, IEE, CEE</t>
+        </is>
+      </c>
       <c r="G313" s="2" t="inlineStr"/>
       <c r="H313" s="2" t="inlineStr">
         <is>
@@ -20231,8 +20354,16 @@
       <c r="L313" s="2" t="n"/>
       <c r="M313" s="2" t="n"/>
       <c r="N313" s="2" t="n"/>
-      <c r="O313" s="2" t="n"/>
-      <c r="P313" s="2" t="n"/>
+      <c r="O313" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P313" s="2" t="inlineStr">
+        <is>
+          <t>1b23QM6y_mF3_yyejrB8E7p2lcZHyTYn4azAECfmtUW8</t>
+        </is>
+      </c>
       <c r="Q313" s="2" t="inlineStr"/>
       <c r="R313" s="2" t="inlineStr"/>
       <c r="S313" s="4" t="inlineStr"/>
@@ -20545,12 +20676,12 @@
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCIONES ACCESIBILIDAD Y EFICIENCIA ENERGÉTICA</t>
+          <t>ENVOLVENTE TÉRMICA/ENERGÉTICA</t>
         </is>
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G319" s="2" t="inlineStr"/>
@@ -20572,7 +20703,7 @@
       </c>
       <c r="P319" s="2" t="inlineStr">
         <is>
-          <t>1ze34d__qQXRS4N97Tf_AilD8O9s0mnlMcB-lHxfPDGM</t>
+          <t>19cE2eC48o4p-wL45C9HXvMvzozwJG8uRo-9kGEfsmiI</t>
         </is>
       </c>
       <c r="Q319" s="2" t="inlineStr"/>
@@ -21262,7 +21393,7 @@
       </c>
       <c r="P331" s="2" t="inlineStr">
         <is>
-          <t>1MJZT8AMgNv4fxUUT_8g0IJjQDnJCNLKF33wHQLEkf6w</t>
+          <t>11FMV_VI4zrBt18HuXTR6iepUobRl2qQjlX9UsvhX3OA</t>
         </is>
       </c>
       <c r="Q331" s="2" t="inlineStr">
@@ -21952,12 +22083,12 @@
       </c>
       <c r="E343" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G343" s="2" t="inlineStr"/>
@@ -22000,7 +22131,7 @@
       </c>
       <c r="P343" s="2" t="inlineStr">
         <is>
-          <t>1nh9_7mfkR60B5p40i52AXTnQde6aB9_C-Owogm7jMD4</t>
+          <t>1VTOzfpmkkdk64GI6bTdeMveLqlfNk2zI9tZ_DIoyipY</t>
         </is>
       </c>
       <c r="Q343" s="2" t="inlineStr"/>
@@ -22856,7 +22987,11 @@
         </is>
       </c>
       <c r="O357" s="2" t="n"/>
-      <c r="P357" s="2" t="n"/>
+      <c r="P357" s="2" t="inlineStr">
+        <is>
+          <t>1qjlNyn-wyVkG_SY-Urgf4KBSsf5z3mHwUOkB9NgkF50</t>
+        </is>
+      </c>
       <c r="Q357" s="2" t="inlineStr">
         <is>
           <t>tanda1 123: RESUELTO LEYENDO: Leída la firmada: 28/05/2026, la versión 'modificado tras reunión' (v2). Mismos importes (proyecto 22.000; subvención 2.500 fijo + 3,5%); cambia el calendario de pagos. CIF con E (comunidad de bienes).</t>
@@ -23327,9 +23462,9 @@
           <t>HE-2026-0365</t>
         </is>
       </c>
-      <c r="B366" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B366" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
@@ -23374,7 +23509,12 @@
           <t>1upXHh26_MmRJYE2zpxw7GlkrCajpa1wY-6zG5hQN2dw</t>
         </is>
       </c>
-      <c r="Q366" s="2" t="inlineStr"/>
+      <c r="Q366" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Misma tramitación de subvenciones con el mismo importe (2.225 + 3,5%), reemitida con número nuevo y pago fraccionado mayo/junio.
+sustituida por: HE-2026-0437</t>
+        </is>
+      </c>
       <c r="R366" s="2" t="inlineStr"/>
       <c r="S366" s="4" t="inlineStr"/>
     </row>
@@ -23384,9 +23524,9 @@
           <t>HE-2026-0366</t>
         </is>
       </c>
-      <c r="B367" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B367" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
@@ -23396,7 +23536,7 @@
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>PASEO PERALES 15 PORTAL 1</t>
+          <t>PASEO PERALES 15 PORTAL 5</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
@@ -23428,10 +23568,15 @@
       </c>
       <c r="P367" s="2" t="inlineStr">
         <is>
-          <t>1upXHh26_MmRJYE2zpxw7GlkrCajpa1wY-6zG5hQN2dw</t>
-        </is>
-      </c>
-      <c r="Q367" s="2" t="inlineStr"/>
+          <t>1LWAIeciVJ0IW5J2iu-nP5mw3rJ-g8n1cBLRzbVLuR60</t>
+        </is>
+      </c>
+      <c r="Q367" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Misma tramitación de subvenciones con documentación técnica 2.225 € para Paseo Perales 15 portal 1, reemitida con pago fraccionado; la posterior se firmó.
+sustituida por: HE-2026-0437</t>
+        </is>
+      </c>
       <c r="R367" s="2" t="inlineStr"/>
       <c r="S367" s="4" t="inlineStr"/>
     </row>
@@ -23545,7 +23690,11 @@
           <t>1mAybcafNpyP_y71J0jbNok4xGiHPoq8Mv0eRaA60Je0</t>
         </is>
       </c>
-      <c r="Q369" s="2" t="inlineStr"/>
+      <c r="Q369" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Mismo proyecto SATE (mismo PEM 490.000/550.000 €) reofertado con formato actual, honorarios 24.010 € y subvención solo a éxito.</t>
+        </is>
+      </c>
       <c r="R369" s="2" t="inlineStr"/>
       <c r="S369" s="4" t="inlineStr"/>
     </row>
@@ -23622,9 +23771,21 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="D371" s="2" t="inlineStr"/>
-      <c r="E371" s="2" t="n"/>
-      <c r="F371" s="2" t="inlineStr"/>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>CALLE 1492 NO 6 SAN SEBASTIÁN DE LOS REYES</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACIÓN ASCENSOR</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+        </is>
+      </c>
       <c r="G371" s="2" t="inlineStr"/>
       <c r="H371" s="2" t="inlineStr">
         <is>
@@ -23637,8 +23798,16 @@
       <c r="L371" s="2" t="n"/>
       <c r="M371" s="2" t="n"/>
       <c r="N371" s="2" t="n"/>
-      <c r="O371" s="2" t="n"/>
-      <c r="P371" s="2" t="n"/>
+      <c r="O371" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P371" s="2" t="inlineStr">
+        <is>
+          <t>16SP1u4fl6-4i7-S8d-2AohD_UUIGKRvJKoMWJDjaNyA</t>
+        </is>
+      </c>
       <c r="Q371" s="2" t="inlineStr"/>
       <c r="R371" s="2" t="inlineStr"/>
       <c r="S371" s="4" t="inlineStr"/>
@@ -24312,9 +24481,21 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="D382" s="2" t="inlineStr"/>
-      <c r="E382" s="2" t="n"/>
-      <c r="F382" s="2" t="inlineStr"/>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALFONSO XII MADRID </t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACION ASC + SUBV</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+        </is>
+      </c>
       <c r="G382" s="2" t="inlineStr"/>
       <c r="H382" s="2" t="inlineStr">
         <is>
@@ -24327,8 +24508,16 @@
       <c r="L382" s="2" t="n"/>
       <c r="M382" s="2" t="n"/>
       <c r="N382" s="2" t="n"/>
-      <c r="O382" s="2" t="n"/>
-      <c r="P382" s="2" t="n"/>
+      <c r="O382" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P382" s="2" t="inlineStr">
+        <is>
+          <t>1mOAHZJnEwXJvpHtzNLRUxKtZPMtKrr5PtG1LUToTWh4</t>
+        </is>
+      </c>
       <c r="Q382" s="2" t="inlineStr"/>
       <c r="R382" s="2" t="inlineStr"/>
       <c r="S382" s="4" t="inlineStr"/>
@@ -25373,12 +25562,12 @@
       </c>
       <c r="E401" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, IEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G401" s="2" t="inlineStr"/>
@@ -25400,7 +25589,7 @@
       </c>
       <c r="P401" s="2" t="inlineStr">
         <is>
-          <t>1nAIN3wjAKsisZpuCpNKBX2aq0BuGUo41xpulTFBN3Ak</t>
+          <t>1gDKoMFPlyKQx8wtGhgiGk_ZuWbK48-x6_HWJiSgySuc</t>
         </is>
       </c>
       <c r="Q401" s="2" t="inlineStr"/>
@@ -25542,16 +25731,8 @@
           <t>ALFREDO ALEIX 44 MADRID</t>
         </is>
       </c>
-      <c r="E404" s="2" t="inlineStr">
-        <is>
-          <t>SATE + CUBIERTA</t>
-        </is>
-      </c>
-      <c r="F404" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="E404" s="2" t="n"/>
+      <c r="F404" s="2" t="inlineStr"/>
       <c r="G404" s="2" t="inlineStr"/>
       <c r="H404" s="2" t="inlineStr">
         <is>
@@ -25564,17 +25745,13 @@
       <c r="L404" s="2" t="n"/>
       <c r="M404" s="2" t="n"/>
       <c r="N404" s="2" t="n"/>
-      <c r="O404" s="2" t="inlineStr">
-        <is>
-          <t>CG/ por alejandra</t>
-        </is>
-      </c>
-      <c r="P404" s="2" t="inlineStr">
-        <is>
-          <t>1g_-QzgdG3OqwBUUJEdA5yfDBK6cyqXyPewxhoZ6KfeQ</t>
-        </is>
-      </c>
-      <c r="Q404" s="2" t="inlineStr"/>
+      <c r="O404" s="2" t="n"/>
+      <c r="P404" s="2" t="n"/>
+      <c r="Q404" s="2" t="inlineStr">
+        <is>
+          <t>id de Drive POR CONFIRMAR: ese día hay 2 hojas de esta dirección en el Excel y el título no casó</t>
+        </is>
+      </c>
       <c r="R404" s="2" t="inlineStr"/>
       <c r="S404" s="4" t="inlineStr"/>
     </row>
@@ -25601,12 +25778,12 @@
       </c>
       <c r="E405" s="2" t="inlineStr">
         <is>
-          <t>SATE + CUBIERTA</t>
+          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F405" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G405" s="2" t="inlineStr"/>
@@ -25628,7 +25805,7 @@
       </c>
       <c r="P405" s="2" t="inlineStr">
         <is>
-          <t>1g_-QzgdG3OqwBUUJEdA5yfDBK6cyqXyPewxhoZ6KfeQ</t>
+          <t>10zp2icqj6YpF5hH6RCsqYw448OT_oZMoDH7au-afLic</t>
         </is>
       </c>
       <c r="Q405" s="2" t="inlineStr"/>
@@ -25742,12 +25919,12 @@
       </c>
       <c r="E407" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G407" s="2" t="inlineStr"/>
@@ -25769,7 +25946,7 @@
       </c>
       <c r="P407" s="2" t="inlineStr">
         <is>
-          <t>1yzUNDmySjCnNnbaqlKuRKFTwUucWLmNStxfTxcWRM-4</t>
+          <t>16ERqkw6DH8CmIdmNs7vKnAotTVhPEYF1OMXxJ5fg_cs</t>
         </is>
       </c>
       <c r="Q407" s="2" t="inlineStr"/>
@@ -25867,12 +26044,12 @@
       </c>
       <c r="E409" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F409" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G409" s="2" t="inlineStr"/>
@@ -25894,7 +26071,7 @@
       </c>
       <c r="P409" s="2" t="inlineStr">
         <is>
-          <t>1mZ0ftLtxtfxhqlAEQZNTprFY-noaE3naKRVMeiIfR0k</t>
+          <t>1QSbNRv06Ndxw7Gi8XhzMRQ4uh81ftM_5vbfMRq7zdIA</t>
         </is>
       </c>
       <c r="Q409" s="2" t="inlineStr"/>
@@ -25981,12 +26158,12 @@
       </c>
       <c r="E411" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F411" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G411" s="2" t="inlineStr"/>
@@ -26008,7 +26185,7 @@
       </c>
       <c r="P411" s="2" t="inlineStr">
         <is>
-          <t>1eWG7YpMfT5BRarzsYJDvRpBHkL8iKClz_SxLR0ZaSPo</t>
+          <t>1q7ZtunZClv0OKz7SLP4FOd_qYVwfV9ORKFdiWg4pPNA</t>
         </is>
       </c>
       <c r="Q411" s="2" t="inlineStr"/>
@@ -26095,12 +26272,12 @@
       </c>
       <c r="E413" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F413" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G413" s="2" t="inlineStr"/>
@@ -26149,7 +26326,7 @@
       </c>
       <c r="P413" s="2" t="inlineStr">
         <is>
-          <t>1DusKT3z6h_XPuaKYkR-gAAdaapEreOAx-xlMapuCuCk</t>
+          <t>1L-1pIm0T_qLh1T3hW9QGqwXb68riUhkGtaBmlDVmTUE</t>
         </is>
       </c>
       <c r="Q413" s="2" t="inlineStr"/>
@@ -26244,9 +26421,9 @@
           <t>HE-2026-0414</t>
         </is>
       </c>
-      <c r="B415" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B415" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C415" s="2" t="inlineStr">
@@ -26291,7 +26468,12 @@
           <t>1av59UUJadsNSxkcI3IGAG1VznW9zC-Lq_woZn9zyKWY</t>
         </is>
       </c>
-      <c r="Q415" s="2" t="inlineStr"/>
+      <c r="Q415" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La 'ascensor + subvenciones' del 21-may se partió al día siguiente en proyecto ascensor (mismo 5.980) y tramitación de subvenciones.
+sustituida por: HE-2026-0426, HE-2026-0427</t>
+        </is>
+      </c>
       <c r="R415" s="2" t="inlineStr"/>
       <c r="S415" s="4" t="inlineStr"/>
     </row>
@@ -26301,9 +26483,9 @@
           <t>HE-2026-0415</t>
         </is>
       </c>
-      <c r="B416" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B416" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C416" s="2" t="inlineStr">
@@ -26348,7 +26530,12 @@
           <t>1RIFs6rH-byiPp-N6VGvhGAmHZawzhEUCiYx5M1YCG_Y</t>
         </is>
       </c>
-      <c r="Q416" s="2" t="inlineStr"/>
+      <c r="Q416" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La tramitación de subvenciones (doc. técnica 1.980 € + 3,5%) se reemitió al día siguiente igual con gestión de subvenciones; el PRY ASCENSOR es encargo aparte.
+sustituida por: HE-2026-0427</t>
+        </is>
+      </c>
       <c r="R416" s="2" t="inlineStr"/>
       <c r="S416" s="4" t="inlineStr"/>
     </row>
@@ -26358,9 +26545,9 @@
           <t>HE-2026-0416</t>
         </is>
       </c>
-      <c r="B417" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B417" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C417" s="2" t="inlineStr">
@@ -26373,16 +26560,8 @@
           <t>GABRIEL USERA 56 MADRID</t>
         </is>
       </c>
-      <c r="E417" s="2" t="inlineStr">
-        <is>
-          <t>INSTALACION ASCENSOR</t>
-        </is>
-      </c>
-      <c r="F417" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="E417" s="2" t="n"/>
+      <c r="F417" s="2" t="inlineStr"/>
       <c r="G417" s="2" t="inlineStr"/>
       <c r="H417" s="2" t="inlineStr">
         <is>
@@ -26395,17 +26574,15 @@
       <c r="L417" s="2" t="n"/>
       <c r="M417" s="2" t="n"/>
       <c r="N417" s="2" t="n"/>
-      <c r="O417" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="P417" s="2" t="inlineStr">
-        <is>
-          <t>1PosldhqjGljtxnxdT6SfP0yWVcOxWpAMVQ30DCVFXXQ</t>
-        </is>
-      </c>
-      <c r="Q417" s="2" t="inlineStr"/>
+      <c r="O417" s="2" t="n"/>
+      <c r="P417" s="2" t="n"/>
+      <c r="Q417" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) El proyecto de SATE/envolvente del 21-may (8.080 €) se fundió al día siguiente con el de ascensor en un único proyecto ascensor + envolvente (14.980 €); la de subvenciones es otro servicio.
+sustituida por: HE-2026-0432
+id de Drive POR CONFIRMAR: ese día hay 3 hojas de esta dirección en el Excel y el título no casó</t>
+        </is>
+      </c>
       <c r="R417" s="2" t="inlineStr"/>
       <c r="S417" s="4" t="inlineStr"/>
     </row>
@@ -26415,9 +26592,9 @@
           <t>HE-2026-0417</t>
         </is>
       </c>
-      <c r="B418" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B418" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C418" s="2" t="inlineStr">
@@ -26462,7 +26639,12 @@
           <t>1PosldhqjGljtxnxdT6SfP0yWVcOxWpAMVQ30DCVFXXQ</t>
         </is>
       </c>
-      <c r="Q418" s="2" t="inlineStr"/>
+      <c r="Q418" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) El proyecto de ascensor (5.980) se reofertó al día siguiente ampliado con envolvente (14.980); la hoja de subvenciones es un encargo añadido que no estaba en la antigua.
+sustituida por: HE-2026-0432</t>
+        </is>
+      </c>
       <c r="R418" s="2" t="inlineStr"/>
       <c r="S418" s="4" t="inlineStr"/>
     </row>
@@ -26472,9 +26654,9 @@
           <t>HE-2026-0418</t>
         </is>
       </c>
-      <c r="B419" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B419" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C419" s="2" t="inlineStr">
@@ -26519,7 +26701,12 @@
           <t>1m2-W-lrtYGAccLxXnTFiRZmi_cyi_9Fb01zagLfJdo8</t>
         </is>
       </c>
-      <c r="Q419" s="2" t="inlineStr"/>
+      <c r="Q419" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) Misma tramitación de subvenciones accesibilidad y EE (1.980 € + 3,5%) reemitida al día siguiente; el PRY ASCENSOR Y SATE es encargo aparte.
+sustituida por: HE-2026-0433</t>
+        </is>
+      </c>
       <c r="R419" s="2" t="inlineStr"/>
       <c r="S419" s="4" t="inlineStr"/>
     </row>
@@ -27053,7 +27240,11 @@
           <t>11Kr_X-XWWg9ll6RVd_fe3FGYGfXuZ6ZixQvYvJcP09w</t>
         </is>
       </c>
-      <c r="Q427" s="2" t="inlineStr"/>
+      <c r="Q427" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La 'ascensor + subvenciones' del 21-may se partió al día siguiente en proyecto ascensor (mismo 5.980) y tramitación de subvenciones.</t>
+        </is>
+      </c>
       <c r="R427" s="2" t="inlineStr"/>
       <c r="S427" s="4" t="inlineStr"/>
     </row>
@@ -27135,7 +27326,12 @@
           <t>1OrekytRpgPAE739b9GmU3PEwtgvUanW4DIxtQAt7UBQ</t>
         </is>
       </c>
-      <c r="Q428" s="2" t="inlineStr"/>
+      <c r="Q428" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La 'ascensor + subvenciones' del 21-may se partió al día siguiente en proyecto ascensor (mismo 5.980) y tramitación de subvenciones.
+sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones (doc. técnica 1.980 € + 3,5%) se reemitió al día siguiente igual con gestión de subvenciones; el PRY ASCENSOR es encargo aparte.</t>
+        </is>
+      </c>
       <c r="R428" s="2" t="inlineStr"/>
       <c r="S428" s="4" t="inlineStr"/>
     </row>
@@ -27220,7 +27416,12 @@
           <t>1CJ1YvRUfdbUnvscFxNMtRmnJKkIMt2-g1li2YPs6Z0I</t>
         </is>
       </c>
-      <c r="Q429" s="2" t="inlineStr"/>
+      <c r="Q429" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de 2 ascensores (8.280, con IEE/CEE) se reofertó ampliado con envolvente (23.000) y el IEE/CEE pasó a la hoja de subvenciones.
+sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de envolvente térmica (con IEE/CEE/libro) se reofertó como proyecto 2 ascensores + envolvente y aparte subvenciones accesibilidad y EE con la documentación técnica; ambas firmadas.</t>
+        </is>
+      </c>
       <c r="R429" s="2" t="inlineStr"/>
       <c r="S429" s="4" t="inlineStr"/>
     </row>
@@ -27304,7 +27505,13 @@
           <t>1WEcZJqfEyHFFHHwOSMamc2Og98e_cMIwZV2g9xdd3V4</t>
         </is>
       </c>
-      <c r="Q430" s="2" t="inlineStr"/>
+      <c r="Q430" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones de accesibilidad y eficiencia del 13-may se rehízo el 22-may (mismo objeto, 1.980 € + 3% a éxito) y es la firmada; el proyecto de 2 ascensores y envolvente es encargo aparte.
+sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de 2 ascensores (8.280, con IEE/CEE) se reofertó ampliado con envolvente (23.000) y el IEE/CEE pasó a la hoja de subvenciones.
+sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de envolvente térmica (con IEE/CEE/libro) se reofertó como proyecto 2 ascensores + envolvente y aparte subvenciones accesibilidad y EE con la documentación técnica; ambas firmadas.</t>
+        </is>
+      </c>
       <c r="R430" s="2" t="inlineStr"/>
       <c r="S430" s="4" t="inlineStr"/>
     </row>
@@ -27388,12 +27595,12 @@
       </c>
       <c r="E432" s="2" t="inlineStr">
         <is>
-          <t>INSTALACION ASCENSOR</t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G432" s="2" t="inlineStr"/>
@@ -27415,7 +27622,7 @@
       </c>
       <c r="P432" s="2" t="inlineStr">
         <is>
-          <t>1Uq4uuvBN3wDrwkFa_CPl323QwLQ9U-08TqukFKg5wNM</t>
+          <t>1OFo6bKzs7AGcgb0B8R2MkKp-2gaY9ECJEzKabTRj7TA</t>
         </is>
       </c>
       <c r="Q432" s="2" t="inlineStr"/>
@@ -27475,7 +27682,12 @@
           <t>1EmsnlVgjgI9jM37p-fH_nXIn-AyJZ2g6x6hBH3AquEg</t>
         </is>
       </c>
-      <c r="Q433" s="2" t="inlineStr"/>
+      <c r="Q433" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de SATE/envolvente del 21-may (8.080 €) se fundió al día siguiente con el de ascensor en un único proyecto ascensor + envolvente (14.980 €); la de subvenciones es otro servicio.
+sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de ascensor (5.980) se reofertó al día siguiente ampliado con envolvente (14.980); la hoja de subvenciones es un encargo añadido que no estaba en la antigua.</t>
+        </is>
+      </c>
       <c r="R433" s="2" t="inlineStr"/>
       <c r="S433" s="4" t="inlineStr"/>
     </row>
@@ -27532,7 +27744,11 @@
           <t>1lNkdNpQjR5WQ-f068S1qPDisdiLmhPDpiYJ2A81XVeE</t>
         </is>
       </c>
-      <c r="Q434" s="2" t="inlineStr"/>
+      <c r="Q434" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Misma tramitación de subvenciones accesibilidad y EE (1.980 € + 3,5%) reemitida al día siguiente; el PRY ASCENSOR Y SATE es encargo aparte.</t>
+        </is>
+      </c>
       <c r="R434" s="2" t="inlineStr"/>
       <c r="S434" s="4" t="inlineStr"/>
     </row>
@@ -27807,7 +28023,12 @@
           <t>17ruZcA1kglzZrkK8f1wpigmXJROrOyYqm-xEN-_dghY</t>
         </is>
       </c>
-      <c r="Q438" s="2" t="inlineStr"/>
+      <c r="Q438" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Misma tramitación de subvenciones con el mismo importe (2.225 + 3,5%), reemitida con número nuevo y pago fraccionado mayo/junio.
+sustituye a la(s) hoja(s) anterior(es): (leído) Misma tramitación de subvenciones con documentación técnica 2.225 € para Paseo Perales 15 portal 1, reemitida con pago fraccionado; la posterior se firmó.</t>
+        </is>
+      </c>
       <c r="R438" s="2" t="inlineStr"/>
       <c r="S438" s="4" t="inlineStr"/>
     </row>
@@ -28347,12 +28568,12 @@
       </c>
       <c r="E448" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA . SATE</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F448" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G448" s="2" t="inlineStr"/>
@@ -28374,7 +28595,7 @@
       </c>
       <c r="P448" s="2" t="inlineStr">
         <is>
-          <t>17pUqMtkKcRdvEsjClf5V4q4ITsvqbfdp9JTiOtJEvbE</t>
+          <t>1v0pzTVofNDgEMPBS3oGCkvkm6Ic_zj5w0kvP1gzEnYQ</t>
         </is>
       </c>
       <c r="Q448" s="2" t="inlineStr"/>
@@ -28489,12 +28710,12 @@
       </c>
       <c r="E450" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TÉRMICA (SATE+CUBIERTA)</t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G450" s="2" t="inlineStr"/>
@@ -28543,7 +28764,7 @@
       </c>
       <c r="P450" s="2" t="inlineStr">
         <is>
-          <t>14QYVYFDx4EmjnxleyoeH2geA03mkpYNKOPMk5lXoboU</t>
+          <t>1czjFfgNKVclW4I33ZqALjVacRSSRHdUQ7sBXIrGDhDs</t>
         </is>
       </c>
       <c r="Q450" s="2" t="inlineStr"/>
@@ -28738,21 +28959,9 @@
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D453" s="2" t="inlineStr">
-        <is>
-          <t>FRANCISCO FATOU 24 MADRID</t>
-        </is>
-      </c>
-      <c r="E453" s="2" t="inlineStr">
-        <is>
-          <t>TRAMITACIÓN SUBVENCIONES</t>
-        </is>
-      </c>
-      <c r="F453" s="2" t="inlineStr">
-        <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
-        </is>
-      </c>
+      <c r="D453" s="2" t="inlineStr"/>
+      <c r="E453" s="2" t="n"/>
+      <c r="F453" s="2" t="inlineStr"/>
       <c r="G453" s="2" t="inlineStr"/>
       <c r="H453" s="2" t="inlineStr">
         <is>
@@ -28765,14 +28974,10 @@
       <c r="L453" s="2" t="n"/>
       <c r="M453" s="2" t="n"/>
       <c r="N453" s="2" t="n"/>
-      <c r="O453" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="O453" s="2" t="n"/>
       <c r="P453" s="2" t="inlineStr">
         <is>
-          <t>1FDGZTUaWR9uMy0Xqfn26j9uQqc8wB-kDS6vJMiAw59s</t>
+          <t>1cgAXSF86u3gFjWDUAkoaARdrXkZ5Ab31-Ns3KCFm94M</t>
         </is>
       </c>
       <c r="Q453" s="2" t="inlineStr"/>
@@ -29055,12 +29260,12 @@
       </c>
       <c r="E458" s="2" t="inlineStr">
         <is>
-          <t>RETIRADA AMIANTO + CUBIERTA</t>
+          <t>TRAMITACION DE SUBVENCIONES</t>
         </is>
       </c>
       <c r="F458" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G458" s="2" t="inlineStr"/>
@@ -29082,7 +29287,7 @@
       </c>
       <c r="P458" s="2" t="inlineStr">
         <is>
-          <t>1MyP5uT2ALFvESNrSLF0vqi83lY-5edEu3RGjE8GGVBc</t>
+          <t>1vsU-wF-bOcb-6HFhg77LxbSpey6QBAs1CHs69ZQdgss</t>
         </is>
       </c>
       <c r="Q458" s="2" t="inlineStr"/>
@@ -29142,7 +29347,11 @@
           <t>1O4R6iaq1rGkwWNuLuzmWZjAeFWM4ZbOxc9ahvA4hOLs</t>
         </is>
       </c>
-      <c r="Q459" s="2" t="inlineStr"/>
+      <c r="Q459" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El PRY ASCENSOR + SUBV de febrero se reofertó en mayo partido en proyecto ascensor y tramitación de subvenciones con IEE/CEE (formato actual).</t>
+        </is>
+      </c>
       <c r="R459" s="2" t="inlineStr"/>
       <c r="S459" s="4" t="inlineStr"/>
     </row>
@@ -29199,7 +29408,11 @@
           <t>1Orx6DTOjvloWRwbN9FlmwY-nCEeSvGKxzoPox-Gz4SI</t>
         </is>
       </c>
-      <c r="Q460" s="2" t="inlineStr"/>
+      <c r="Q460" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El PRY ASCENSOR + SUBV de febrero se reofertó en mayo partido en proyecto ascensor y tramitación de subvenciones con IEE/CEE (formato actual).</t>
+        </is>
+      </c>
       <c r="R460" s="2" t="inlineStr"/>
       <c r="S460" s="4" t="inlineStr"/>
     </row>
@@ -29256,7 +29469,11 @@
           <t>1kGJG_7bBwm7LaxFfZYiJRKOLFFBW2W0VGLHvDUVq3Oc</t>
         </is>
       </c>
-      <c r="Q461" s="2" t="inlineStr"/>
+      <c r="Q461" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de ascensor + subvención accesibilidad de febrero se renovó en mayo partido en proyecto de ascensor (+CSS) y tramitación de subvenciones con el formato actual.</t>
+        </is>
+      </c>
       <c r="R461" s="2" t="inlineStr"/>
       <c r="S461" s="4" t="inlineStr"/>
     </row>
@@ -29313,7 +29530,11 @@
           <t>19wz0kmWoGb19GvzCTAFgPNw43b4b-wbLuj5bGuATMrQ</t>
         </is>
       </c>
-      <c r="Q462" s="2" t="inlineStr"/>
+      <c r="Q462" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) El proyecto de ascensor + subvención accesibilidad de febrero se renovó en mayo partido en proyecto de ascensor (+CSS) y tramitación de subvenciones con el formato actual.</t>
+        </is>
+      </c>
       <c r="R462" s="2" t="inlineStr"/>
       <c r="S462" s="4" t="inlineStr"/>
     </row>
@@ -29965,12 +30186,12 @@
       </c>
       <c r="E473" s="2" t="inlineStr">
         <is>
-          <t>IMPERMIABILIZACIÓN Y AISLAMIENTO TERMICO INCLUYENDO RETIRADA DE URALITA</t>
+          <t>ACCESIBILIDAD CON PLATAFORMA ELEVADORA VERTICAL</t>
         </is>
       </c>
       <c r="F473" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G473" s="2" t="inlineStr"/>
@@ -29992,7 +30213,7 @@
       </c>
       <c r="P473" s="2" t="inlineStr">
         <is>
-          <t>1XT1rAcyAJmyGwmVcs9pYsvayOAJYzD0XkmQls5xbnRg</t>
+          <t>1Wfzm9_XaVdZqEefVyJ-enFLsvDD7N2sUSZxbdTU9vKY</t>
         </is>
       </c>
       <c r="Q473" s="2" t="inlineStr"/>
@@ -30077,16 +30298,8 @@
           <t>CASTELLO 106 MADRID</t>
         </is>
       </c>
-      <c r="E475" s="2" t="inlineStr">
-        <is>
-          <t>IMPERMIABILIZACIÓN Y AISLAMIENTO TERMICO INCLUYENDO RETIRADA DE URALITA</t>
-        </is>
-      </c>
-      <c r="F475" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="E475" s="2" t="n"/>
+      <c r="F475" s="2" t="inlineStr"/>
       <c r="G475" s="2" t="inlineStr"/>
       <c r="H475" s="2" t="inlineStr">
         <is>
@@ -30099,17 +30312,13 @@
       <c r="L475" s="2" t="n"/>
       <c r="M475" s="2" t="n"/>
       <c r="N475" s="2" t="n"/>
-      <c r="O475" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="P475" s="2" t="inlineStr">
-        <is>
-          <t>1XT1rAcyAJmyGwmVcs9pYsvayOAJYzD0XkmQls5xbnRg</t>
-        </is>
-      </c>
-      <c r="Q475" s="2" t="inlineStr"/>
+      <c r="O475" s="2" t="n"/>
+      <c r="P475" s="2" t="n"/>
+      <c r="Q475" s="2" t="inlineStr">
+        <is>
+          <t>id de Drive POR CONFIRMAR: ese día hay 4 hojas de esta dirección en el Excel y el título no casó</t>
+        </is>
+      </c>
       <c r="R475" s="2" t="inlineStr"/>
       <c r="S475" s="4" t="inlineStr"/>
     </row>
@@ -30136,12 +30345,12 @@
       </c>
       <c r="E476" s="2" t="inlineStr">
         <is>
-          <t>IMPERMIABILIZACIÓN Y AISLAMIENTO TERMICO INCLUYENDO RETIRADA DE URALITA</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F476" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G476" s="2" t="inlineStr"/>
@@ -30163,7 +30372,7 @@
       </c>
       <c r="P476" s="2" t="inlineStr">
         <is>
-          <t>1XT1rAcyAJmyGwmVcs9pYsvayOAJYzD0XkmQls5xbnRg</t>
+          <t>145dBeMPpQPj3fqff1TnqzqtsT7h85IZbR_w_cj02qIg</t>
         </is>
       </c>
       <c r="Q476" s="2" t="inlineStr"/>
@@ -30364,12 +30573,12 @@
       </c>
       <c r="E480" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F480" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G480" s="2" t="inlineStr"/>
@@ -30391,7 +30600,7 @@
       </c>
       <c r="P480" s="2" t="inlineStr">
         <is>
-          <t>1TrHL3EmjTBK8fLGfhKaWUzpHhzZXUQPx_10UQsltd8M</t>
+          <t>1GXlRCgf27kiPpLOGGMjlAjlJbCRuGixP1TNmgUKTwv8</t>
         </is>
       </c>
       <c r="Q480" s="2" t="inlineStr"/>
@@ -30706,12 +30915,12 @@
       </c>
       <c r="E486" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
+          <t>ENVOLVENTE TERMICA ( SATE )</t>
         </is>
       </c>
       <c r="F486" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G486" s="2" t="inlineStr"/>
@@ -30733,7 +30942,7 @@
       </c>
       <c r="P486" s="2" t="inlineStr">
         <is>
-          <t>1V7ipskRPXuNrA0n1IfkLlWFWjO1BNadQeCMIzwpKfQQ</t>
+          <t>1LhK4Po8bcZ_SNBOKp14GbU9u2-DzljAj0LMlZT4Q3gg</t>
         </is>
       </c>
       <c r="Q486" s="2" t="inlineStr"/>
@@ -30820,12 +31029,12 @@
       </c>
       <c r="E488" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F488" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G488" s="2" t="inlineStr"/>
@@ -30847,7 +31056,7 @@
       </c>
       <c r="P488" s="2" t="inlineStr">
         <is>
-          <t>1ajgQDv8jH4_3bSjv1CO7ZBzrubZwT9i6yZBnANskMVs</t>
+          <t>1UXl3gyEzUGUCe69zn4pifCkjK3ca-MhzB_zRdlpnIo8</t>
         </is>
       </c>
       <c r="Q488" s="2" t="inlineStr"/>
@@ -31957,12 +32166,12 @@
       </c>
       <c r="E507" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F507" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G507" s="2" t="inlineStr"/>
@@ -31984,7 +32193,7 @@
       </c>
       <c r="P507" s="2" t="inlineStr">
         <is>
-          <t>1vs72uuCXQ3urZ1N3NVyeUnq6yhjqOPpmw3aYt9Y68Y4</t>
+          <t>1ztQY25uRlJXBefLnvevkZnsaL0jJ8SQPX-HL_yfMvcI</t>
         </is>
       </c>
       <c r="Q507" s="2" t="inlineStr"/>
@@ -32111,9 +32320,9 @@
           <t>HE-2026-0509</t>
         </is>
       </c>
-      <c r="B510" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B510" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C510" s="2" t="inlineStr">
@@ -32128,12 +32337,12 @@
       </c>
       <c r="E510" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR CON DERRIBO DE ESCALERA</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F510" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G510" s="2" t="inlineStr"/>
@@ -32155,10 +32364,15 @@
       </c>
       <c r="P510" s="2" t="inlineStr">
         <is>
-          <t>13_a2-qqOnmhNKxGxv-hbmhEd_j3T3HaCdYQM1CZOS3E</t>
-        </is>
-      </c>
-      <c r="Q510" s="2" t="inlineStr"/>
+          <t>1wTfQGhUMTYCAnrZy1bxsi5---dPsRiAC5GhTi_xDiq0</t>
+        </is>
+      </c>
+      <c r="Q510" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La tramitación de subvenciones de accesibilidad del 8-jun se reenvió idéntica (1.980 € + 3,5% a éxito) el 20-jun junto al proyecto de ascensor renovado.
+sustituida por: HE-2026-0554</t>
+        </is>
+      </c>
       <c r="R510" s="2" t="inlineStr"/>
       <c r="S510" s="4" t="inlineStr"/>
     </row>
@@ -32242,12 +32456,12 @@
       </c>
       <c r="E512" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F512" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G512" s="2" t="inlineStr"/>
@@ -32269,7 +32483,7 @@
       </c>
       <c r="P512" s="2" t="inlineStr">
         <is>
-          <t>1weu1bFh2gcij48ieBWcLSyTlevtvsuVkLvp-1z50WTk</t>
+          <t>11l44ucXWyPHiPRihC-CfqJTiU-8MZiYbYql2OvQpogI</t>
         </is>
       </c>
       <c r="Q512" s="2" t="inlineStr"/>
@@ -32356,12 +32570,12 @@
       </c>
       <c r="E514" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA ( SATE )</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F514" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G514" s="2" t="inlineStr"/>
@@ -32383,7 +32597,7 @@
       </c>
       <c r="P514" s="2" t="inlineStr">
         <is>
-          <t>1xx6rHYpPQ_kjKJ4VMCiFjSki5_wtBXdaphuQhD8napU</t>
+          <t>1ZZWNhTkkCrJerZ19eloIsWb6_vVUPWq-AxZnvGHNVT0</t>
         </is>
       </c>
       <c r="Q514" s="2" t="inlineStr"/>
@@ -33040,12 +33254,12 @@
       </c>
       <c r="E526" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA ( SATE )</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F526" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G526" s="2" t="inlineStr"/>
@@ -33067,7 +33281,7 @@
       </c>
       <c r="P526" s="2" t="inlineStr">
         <is>
-          <t>1ovuLw93dgZvdXiHL584dNGJPve1kgjeWDLmdzxm7Q1s</t>
+          <t>11RIvMkh7VEzC4DQOoY-DzGgI28TtH7y0IP4QLBIWd3s</t>
         </is>
       </c>
       <c r="Q526" s="2" t="inlineStr"/>
@@ -33496,12 +33710,12 @@
       </c>
       <c r="E534" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F534" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G534" s="2" t="inlineStr"/>
@@ -33523,7 +33737,7 @@
       </c>
       <c r="P534" s="2" t="inlineStr">
         <is>
-          <t>1bz4EuIDv9DfxcdOQEfJfW9vFU2Bb81DhkC5YTJh2FhE</t>
+          <t>1Mk_kqlpLYAuor5IxCeDwpDJATGT7ZCag0PefaZeTkOY</t>
         </is>
       </c>
       <c r="Q534" s="2" t="inlineStr"/>
@@ -34333,9 +34547,9 @@
           <t>HE-2026-0547</t>
         </is>
       </c>
-      <c r="B548" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B548" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C548" s="2" t="inlineStr">
@@ -34380,7 +34594,12 @@
           <t>1rplkHTvlQ8QXye9Q9UvpEUNZDy6rLPXMQVSTPKTbHNA</t>
         </is>
       </c>
-      <c r="Q548" s="2" t="inlineStr"/>
+      <c r="Q548" s="2" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA: (leído) La subvención 'para proyecto externo' (2.625) se reofertó como tramitación de subvenciones normal (1.980) al encargar también el proyecto de ascensor, que es un encargo nuevo.
+sustituida por: HE-2026-0567</t>
+        </is>
+      </c>
       <c r="R548" s="2" t="inlineStr"/>
       <c r="S548" s="4" t="inlineStr"/>
     </row>
@@ -34464,12 +34683,12 @@
       </c>
       <c r="E550" s="2" t="inlineStr">
         <is>
-          <t>ACCESIBILIDAD</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F550" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G550" s="2" t="inlineStr"/>
@@ -34491,7 +34710,7 @@
       </c>
       <c r="P550" s="2" t="inlineStr">
         <is>
-          <t>1VbiJadDVW5b5pf7_5XmSgF7Zca_cazkm-UsQjBBnOS0</t>
+          <t>1DoSkzbRjTDkXuBxHe5GilMOgd94vCWP6p92CdWGIie4</t>
         </is>
       </c>
       <c r="Q550" s="2" t="inlineStr"/>
@@ -34806,7 +35025,11 @@
           <t>1Fowm4Lr-LCLhv0dufgUJd3ToufK2Q0yHepPBcJSD40Q</t>
         </is>
       </c>
-      <c r="Q555" s="2" t="inlineStr"/>
+      <c r="Q555" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones de accesibilidad del 8-jun se reenvió idéntica (1.980 € + 3,5% a éxito) el 20-jun junto al proyecto de ascensor renovado.</t>
+        </is>
+      </c>
       <c r="R555" s="2" t="inlineStr"/>
       <c r="S555" s="4" t="inlineStr"/>
     </row>
@@ -35593,7 +35816,11 @@
           <t>1ce8PX9oOgX_jhPkP6tT8v-beFlLHt2nvfdlkuTQ8xeQ</t>
         </is>
       </c>
-      <c r="Q568" s="2" t="inlineStr"/>
+      <c r="Q568" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La subvención 'para proyecto externo' (2.625) se reofertó como tramitación de subvenciones normal (1.980) al encargar también el proyecto de ascensor, que es un encargo nuevo.</t>
+        </is>
+      </c>
       <c r="R568" s="2" t="inlineStr"/>
       <c r="S568" s="4" t="inlineStr"/>
     </row>
@@ -35899,7 +36126,14 @@
           <t>1mDbnsOxikYiJ0c2G1Jxo_njPP029_ui06Ka1Ep5QCh8</t>
         </is>
       </c>
-      <c r="Q573" s="2" t="inlineStr"/>
+      <c r="Q573" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones de accesibilidad del portal 1 (765 € fijo) se reofertó a los portales 1-2-3 juntos en junio, hoja firmada.
+sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones de accesibilidad del portal 3 (765 € fijo) se reofertó a los portales 1-2-3 juntos en junio, hoja firmada.
+sustituye a la(s) hoja(s) anterior(es): (leído) Misma tramitación de subvenciones de accesibilidad del portal 1, reofertada a los portales 1-2-3 con el formato actual (doc. técnica 2.625 + 3,5%).
+sustituye a la(s) hoja(s) anterior(es): (leído) La tramitación de subvenciones de accesibilidad del portal se reofertó para los portales 1-2-3 (mancomunidad) con IEE/CEE; la posterior se firmó.</t>
+        </is>
+      </c>
       <c r="R573" s="2" t="inlineStr"/>
       <c r="S573" s="4" t="inlineStr"/>
     </row>
@@ -36036,12 +36270,12 @@
       </c>
       <c r="E576" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA (SATE )</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F576" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G576" s="2" t="inlineStr"/>
@@ -36056,10 +36290,14 @@
       <c r="L576" s="2" t="n"/>
       <c r="M576" s="2" t="n"/>
       <c r="N576" s="2" t="n"/>
-      <c r="O576" s="2" t="n"/>
+      <c r="O576" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="P576" s="2" t="inlineStr">
         <is>
-          <t>1hYrT5a0IEpdXKN-UC34Q6_KUcEhSKG9LG15N0U9Geow</t>
+          <t>1uzt3VMT1HqIRnWpqpovsjoeFDaqU4j88oI3aaFzDtjA</t>
         </is>
       </c>
       <c r="Q576" s="2" t="inlineStr"/>
@@ -36146,12 +36384,12 @@
       </c>
       <c r="E578" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA (SATE + CUBIERTA)</t>
+          <t xml:space="preserve">TRAMITACION DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F578" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G578" s="2" t="inlineStr"/>
@@ -36173,7 +36411,7 @@
       </c>
       <c r="P578" s="2" t="inlineStr">
         <is>
-          <t>1Tc71Mj7iDQ_24h64NvWKishdsacVuyttsuOQSX-tWSU</t>
+          <t>1rePWKftr5-iL6tkjw8BSelCuBffgRReczKMKU33-3i4</t>
         </is>
       </c>
       <c r="Q578" s="2" t="inlineStr"/>
@@ -37354,12 +37592,12 @@
       </c>
       <c r="E599" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACCESIBILIDAD DE JARDIN </t>
+          <t xml:space="preserve">TRAMITACIÓN SUBVENCIONES ACCESIBILIDAD </t>
         </is>
       </c>
       <c r="F599" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G599" s="2" t="inlineStr"/>
@@ -37381,7 +37619,7 @@
       </c>
       <c r="P599" s="2" t="inlineStr">
         <is>
-          <t>16GbdeKd9ILCMZbKn2ZBo2dKWnOr8D4odGw4Eu9XQRyM</t>
+          <t>1elteEgVNEtL-AmpeE50ce-8zVmedZogL05P2LL7u3yw</t>
         </is>
       </c>
       <c r="Q599" s="2" t="inlineStr"/>
@@ -38150,8 +38388,16 @@
           <t>PASEO DE LA HABANA 80 MADRID</t>
         </is>
       </c>
-      <c r="E613" s="2" t="n"/>
-      <c r="F613" s="2" t="inlineStr"/>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENVOLVENTE TERMICA ( SATE ) + ACCESIBILIDAD </t>
+        </is>
+      </c>
+      <c r="F613" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G613" s="2" t="inlineStr"/>
       <c r="H613" s="2" t="inlineStr">
         <is>
@@ -38192,8 +38438,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O613" s="2" t="n"/>
-      <c r="P613" s="2" t="n"/>
+      <c r="O613" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P613" s="2" t="inlineStr">
+        <is>
+          <t>1IkqRm1jVEMDs6FPvyPJJNY5uQi5XplJKFCO2c7XdmVI</t>
+        </is>
+      </c>
       <c r="Q613" s="2" t="inlineStr"/>
       <c r="R613" s="2" t="inlineStr"/>
       <c r="S613" s="4" t="inlineStr"/>
@@ -38614,12 +38868,12 @@
       </c>
       <c r="E620" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENVOLVENTE TERMICA (SATE) </t>
+          <t xml:space="preserve">TRAMITACIÓN DE SUBVENCIONES </t>
         </is>
       </c>
       <c r="F620" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G620" s="2" t="inlineStr"/>
@@ -38641,7 +38895,7 @@
       </c>
       <c r="P620" s="2" t="inlineStr">
         <is>
-          <t>1uGMjdNqSBrqJe5HBLgllRTGRUSfy5cP_s9iPhV2cegQ</t>
+          <t>1PfSdyKqbpaacJvfoT967Tru_lAYd7ogGLhiLkhVtt_Q</t>
         </is>
       </c>
       <c r="Q620" s="2" t="inlineStr"/>
@@ -38758,7 +39012,11 @@
           <t>1p2A1GR9P0YrMpP7c1xNl9Nt4EQqOhjRulrZQz141pPs</t>
         </is>
       </c>
-      <c r="Q622" s="2" t="inlineStr"/>
+      <c r="Q622" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Proyecto de ascensor + subvención accesibilidad de marzo renovado en julio separado en proyecto de ascensor (+CSS, pago fraccionado) y tramitación de subvenciones de accesibilidad.</t>
+        </is>
+      </c>
       <c r="R622" s="2" t="inlineStr"/>
       <c r="S622" s="4" t="inlineStr"/>
     </row>
@@ -38815,7 +39073,11 @@
           <t>1-pUND9EjWW8ShHtOnDGd__ryH5hYY1F2GS268kTxjdk</t>
         </is>
       </c>
-      <c r="Q623" s="2" t="inlineStr"/>
+      <c r="Q623" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) Proyecto de ascensor + subvención accesibilidad de marzo renovado en julio separado en proyecto de ascensor (+CSS, pago fraccionado) y tramitación de subvenciones de accesibilidad.</t>
+        </is>
+      </c>
       <c r="R623" s="2" t="inlineStr"/>
       <c r="S623" s="4" t="inlineStr"/>
     </row>
@@ -39127,12 +39389,12 @@
       </c>
       <c r="E629" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F629" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G629" s="2" t="inlineStr"/>
@@ -39154,7 +39416,7 @@
       </c>
       <c r="P629" s="2" t="inlineStr">
         <is>
-          <t>15hJxxZf4V4r-u-6LkTDm5w1py1OC79gURLG-x7DTZ2g</t>
+          <t>1JgBvRxQKCMkL5UqxzofFpsKPzyjgXwoKkspVOyNvdn0</t>
         </is>
       </c>
       <c r="Q629" s="2" t="inlineStr"/>
@@ -39241,12 +39503,12 @@
       </c>
       <c r="E631" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F631" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G631" s="2" t="inlineStr"/>
@@ -39268,7 +39530,7 @@
       </c>
       <c r="P631" s="2" t="inlineStr">
         <is>
-          <t>1ipbfOZ8jNThIbdBmYQ6XBOh59kXFsrZ7fFG46joO8As</t>
+          <t>1Re4Djdnza1IAAfyT1A6K8pNS59B5jn1j7oWAjmzrnSs</t>
         </is>
       </c>
       <c r="Q631" s="2" t="inlineStr"/>
@@ -39291,21 +39553,9 @@
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D632" s="2" t="inlineStr">
-        <is>
-          <t>PASEO DE EXTREMADURA 150 MADRID</t>
-        </is>
-      </c>
-      <c r="E632" s="2" t="inlineStr">
-        <is>
-          <t>CUBIERTA</t>
-        </is>
-      </c>
-      <c r="F632" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="D632" s="2" t="inlineStr"/>
+      <c r="E632" s="2" t="n"/>
+      <c r="F632" s="2" t="inlineStr"/>
       <c r="G632" s="2" t="inlineStr"/>
       <c r="H632" s="2" t="inlineStr">
         <is>
@@ -39318,14 +39568,10 @@
       <c r="L632" s="2" t="n"/>
       <c r="M632" s="2" t="n"/>
       <c r="N632" s="2" t="n"/>
-      <c r="O632" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O632" s="2" t="n"/>
       <c r="P632" s="2" t="inlineStr">
         <is>
-          <t>1ZwjbrSuzriGAAo7E_k42xFiYBtJ9GOoNgEYbSILA_Ao</t>
+          <t>11BkEvAG3VA5rkxbiThAx4MIY5rQ97TK1j9BCZXmdTvU</t>
         </is>
       </c>
       <c r="Q632" s="2" t="inlineStr"/>
@@ -39412,12 +39658,12 @@
       </c>
       <c r="E634" s="2" t="inlineStr">
         <is>
-          <t>CUBIERTA</t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F634" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G634" s="2" t="inlineStr"/>
@@ -39439,7 +39685,7 @@
       </c>
       <c r="P634" s="2" t="inlineStr">
         <is>
-          <t>1ZwjbrSuzriGAAo7E_k42xFiYBtJ9GOoNgEYbSILA_Ao</t>
+          <t>14uF2lvjwgWL4fTuG1f7FBJ0eQGlmUEIbEpSjkEcU5gU</t>
         </is>
       </c>
       <c r="Q634" s="2" t="inlineStr"/>
@@ -39701,7 +39947,11 @@
       <c r="M638" s="2" t="n"/>
       <c r="N638" s="2" t="n"/>
       <c r="O638" s="2" t="n"/>
-      <c r="P638" s="2" t="n"/>
+      <c r="P638" s="2" t="inlineStr">
+        <is>
+          <t>1176EcJDRLC8K5CqhYcM-X1ezV_mbdUIRcxtARP7NomM</t>
+        </is>
+      </c>
       <c r="Q638" s="2" t="inlineStr"/>
       <c r="R638" s="2" t="inlineStr"/>
       <c r="S638" s="4" t="inlineStr"/>
@@ -39722,9 +39972,21 @@
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="D639" s="2" t="inlineStr"/>
-      <c r="E639" s="2" t="n"/>
-      <c r="F639" s="2" t="inlineStr"/>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SERRANO ORIVE 1 MADRID</t>
+        </is>
+      </c>
+      <c r="E639" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACIÓN ASCENSOR</t>
+        </is>
+      </c>
+      <c r="F639" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G639" s="2" t="inlineStr"/>
       <c r="H639" s="2" t="inlineStr">
         <is>
@@ -39737,8 +39999,16 @@
       <c r="L639" s="2" t="n"/>
       <c r="M639" s="2" t="n"/>
       <c r="N639" s="2" t="n"/>
-      <c r="O639" s="2" t="n"/>
-      <c r="P639" s="2" t="n"/>
+      <c r="O639" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P639" s="2" t="inlineStr">
+        <is>
+          <t>1oGsJA2ozK6Tn396GHoh5SIjg-vKJcmmv-Z6m3RuPoX0</t>
+        </is>
+      </c>
       <c r="Q639" s="2" t="inlineStr"/>
       <c r="R639" s="2" t="inlineStr"/>
       <c r="S639" s="4" t="inlineStr"/>
@@ -39796,7 +40066,11 @@
           <t>1IZ3R38MYPAZYxOtAuqwpn9LlOXpQHDJjPuGruOr8mtA</t>
         </is>
       </c>
-      <c r="Q640" s="2" t="inlineStr"/>
+      <c r="Q640" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La de enero (envolvente/SATE + subvención eficiencia energética + CAES, 8.500 €) se reofertó en julio partida en proyecto SATE+CSS y tramitación de subvenciones de eficiencia; el elevador con derribo y la subvención de accesibilidad de septiembre son otro encargo.</t>
+        </is>
+      </c>
       <c r="R640" s="2" t="inlineStr"/>
       <c r="S640" s="4" t="inlineStr"/>
     </row>
@@ -39823,12 +40097,12 @@
       </c>
       <c r="E641" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENVOLVENTE TERMICA (SATE) </t>
+          <t>TRAMITACIÓN SUBVENCIONES</t>
         </is>
       </c>
       <c r="F641" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G641" s="2" t="inlineStr"/>
@@ -39850,12 +40124,12 @@
       </c>
       <c r="P641" s="2" t="inlineStr">
         <is>
-          <t>1IZ3R38MYPAZYxOtAuqwpn9LlOXpQHDJjPuGruOr8mtA</t>
+          <t>120U9DZaQ0QiIVG_vW9QhqMbpNGxt42uWs23qGNzF4NM</t>
         </is>
       </c>
       <c r="Q641" s="2" t="inlineStr">
         <is>
-          <t>hoja distinta, no versión (leído): Obras distintas: la de julio es proyecto de envolvente térmica (SATE) y la de septiembre instalación de elevador con derribo de escalera.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): (leído) La de enero (envolvente/SATE + subvención eficiencia energética + CAES, 8.500 €) se reofertó en julio partida en proyecto SATE+CSS y tramitación de subvenciones de eficiencia; el elevador con derribo y la subvención de accesibilidad de septiembre son otro encargo.</t>
         </is>
       </c>
       <c r="R641" s="2" t="inlineStr"/>
@@ -40637,8 +40911,16 @@
           <t>HONDURAS 20 COSLADA</t>
         </is>
       </c>
-      <c r="E654" s="2" t="n"/>
-      <c r="F654" s="2" t="inlineStr"/>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFORME DE INSTALACIÓN DE 2 ASCENSORES Y ASESORAMIENTO SOBRE SUBVENCIONES </t>
+        </is>
+      </c>
+      <c r="F654" s="2" t="inlineStr">
+        <is>
+          <t>INFORME PERICIAL</t>
+        </is>
+      </c>
       <c r="G654" s="2" t="inlineStr"/>
       <c r="H654" s="2" t="inlineStr">
         <is>
@@ -40674,8 +40956,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O654" s="2" t="n"/>
-      <c r="P654" s="2" t="n"/>
+      <c r="O654" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P654" s="2" t="inlineStr">
+        <is>
+          <t>1BQovcX8b2-jTjwU7Oy18zLZg85o43gdn0QY1ffzRDQw</t>
+        </is>
+      </c>
       <c r="Q654" s="2" t="inlineStr">
         <is>
           <t>tanda1 133: RESUELTO LEYENDO: El asesoramiento sobre ayudas va incluido en el precio del informe: no es línea aparte.</t>
@@ -41185,7 +41475,7 @@
       </c>
       <c r="E663" s="2" t="inlineStr">
         <is>
-          <t>PROYECTO SATE CUBIERTA Y FACHADA // ACCESIBILIDAD RAMPA</t>
+          <t>SATE CUBIERTA Y FACHADA</t>
         </is>
       </c>
       <c r="F663" s="2" t="inlineStr">
@@ -41212,7 +41502,7 @@
       </c>
       <c r="P663" s="2" t="inlineStr">
         <is>
-          <t>1zpuunNNoSHXwE2j694JQB3YtVSG6ClkTAmcYLzFf0jI</t>
+          <t>10nbql3ujbs9t4hM5Kw47ZGWZSAdwIxH60SRP-2cW68U</t>
         </is>
       </c>
       <c r="Q663" s="2" t="inlineStr"/>
@@ -41299,12 +41589,12 @@
       </c>
       <c r="E665" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCIONES ACCESIBILIDAD</t>
+          <t>SUBVENCIONES EFICIENCIA ENERGÉTICA</t>
         </is>
       </c>
       <c r="F665" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G665" s="2" t="inlineStr"/>
@@ -41326,7 +41616,7 @@
       </c>
       <c r="P665" s="2" t="inlineStr">
         <is>
-          <t>1-NZDkLmghXhcjUh0E_R_nkIMXCQU0I26R-iogip7A9E</t>
+          <t>1-9pdFhz_ZGxMu6WvG6-LGbWXPOEQzNOsNPGpjZ70i14</t>
         </is>
       </c>
       <c r="Q665" s="2" t="inlineStr"/>
@@ -41356,12 +41646,12 @@
       </c>
       <c r="E666" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCIONES EFICIENCIA ENERGÉTICA</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F666" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G666" s="2" t="inlineStr"/>
@@ -41383,7 +41673,7 @@
       </c>
       <c r="P666" s="2" t="inlineStr">
         <is>
-          <t>1-9pdFhz_ZGxMu6WvG6-LGbWXPOEQzNOsNPGpjZ70i14</t>
+          <t>1-NZDkLmghXhcjUh0E_R_nkIMXCQU0I26R-iogip7A9E</t>
         </is>
       </c>
       <c r="Q666" s="2" t="inlineStr"/>
@@ -41584,12 +41874,12 @@
       </c>
       <c r="E670" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA (SATE )</t>
+          <t>SUBVENCIONES EFICIENCIA ENERGÉTICA</t>
         </is>
       </c>
       <c r="F670" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G670" s="2" t="inlineStr"/>
@@ -41611,7 +41901,7 @@
       </c>
       <c r="P670" s="2" t="inlineStr">
         <is>
-          <t>1Hk9HeoSx7sMNGqTEory5S-5JPuJTPkPplGwRyumut7I</t>
+          <t>1rbOEw2wrknHj7mL0Qtt3bZlftE8syVMZlNhXaSnpg-o</t>
         </is>
       </c>
       <c r="Q670" s="2" t="inlineStr"/>
@@ -41983,12 +42273,12 @@
       </c>
       <c r="E677" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TERMICA (SATE )</t>
+          <t>SUBVENCIONES EFICIENCIA ENERGÉTICA</t>
         </is>
       </c>
       <c r="F677" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G677" s="2" t="inlineStr"/>
@@ -42010,7 +42300,7 @@
       </c>
       <c r="P677" s="2" t="inlineStr">
         <is>
-          <t>1FHXDAVRVAqyh8Sg9A1fWECfp_nEE-C8gzKBLtDFHmVQ</t>
+          <t>1_hYtlBDlQbW8LSvWVbRRGI-lDORHDknh33WxExsKCvs</t>
         </is>
       </c>
       <c r="Q677" s="2" t="inlineStr"/>
@@ -42154,7 +42444,7 @@
       </c>
       <c r="E680" s="2" t="inlineStr">
         <is>
-          <t>PRY CONJUNTO ACCESIBILIDAD Y SATE</t>
+          <t>ENVOLVENTE TÉRMICA (SATE)</t>
         </is>
       </c>
       <c r="F680" s="2" t="inlineStr">
@@ -42181,7 +42471,7 @@
       </c>
       <c r="P680" s="2" t="inlineStr">
         <is>
-          <t>1QAyzEqSzjKq9MdOjTuP_p1xgU_Egxv2Kx30aS8dcyNI</t>
+          <t>1QOWWz6rapsUanuFs9Y4Ije-CXdW8Fz_xaunb49Zt_Dw</t>
         </is>
       </c>
       <c r="Q680" s="2" t="inlineStr"/>
@@ -42211,12 +42501,12 @@
       </c>
       <c r="E681" s="2" t="inlineStr">
         <is>
-          <t>PRY CONJUNTO ACCESIBILIDAD Y SATE</t>
+          <t>SUBVENCIONES ACCESIBILIDAD Y EFICIENCIA ENERGÉTICA</t>
         </is>
       </c>
       <c r="F681" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G681" s="2" t="inlineStr"/>
@@ -42238,7 +42528,7 @@
       </c>
       <c r="P681" s="2" t="inlineStr">
         <is>
-          <t>1QAyzEqSzjKq9MdOjTuP_p1xgU_Egxv2Kx30aS8dcyNI</t>
+          <t>1JOeui4R9_o0YJDpTDIRAFU_A174FV4vT4U_z-B-KlUs</t>
         </is>
       </c>
       <c r="Q681" s="2" t="inlineStr"/>
@@ -42268,12 +42558,12 @@
       </c>
       <c r="E682" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCIONES ACCESIBILIDAD Y EFICIENCIA ENERGÉTICA</t>
+          <t>SUBVENCIONAS ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F682" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G682" s="2" t="inlineStr"/>
@@ -42295,7 +42585,7 @@
       </c>
       <c r="P682" s="2" t="inlineStr">
         <is>
-          <t>1JOeui4R9_o0YJDpTDIRAFU_A174FV4vT4U_z-B-KlUs</t>
+          <t>1fEHQTFBxk-vf6AqRtkiMPBTkEdcHZ0xt9I_MDPnXAlI</t>
         </is>
       </c>
       <c r="Q682" s="2" t="inlineStr"/>
@@ -42938,12 +43228,12 @@
       </c>
       <c r="E693" s="2" t="inlineStr">
         <is>
-          <t>ENVOLVENTE TÉRMICA (SATE ) PARA FACHADA Y CUBIERTA</t>
+          <t>SUBVENCIÓN EFICIENCIA ENERGÉTICA PARA PROYECTO REALIZADO POR ACCESALIA</t>
         </is>
       </c>
       <c r="F693" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, IEE, LEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA</t>
         </is>
       </c>
       <c r="G693" s="2" t="inlineStr"/>
@@ -42965,7 +43255,7 @@
       </c>
       <c r="P693" s="2" t="inlineStr">
         <is>
-          <t>1Kl0HTIwaUjoRFvKjoKDtNPEwHEeMyNbnKeHuN1oScnY</t>
+          <t>13tF2CHpdoFeJyddSYNuYf9O884EU-I0KQ1P0ZVJeaZo</t>
         </is>
       </c>
       <c r="Q693" s="2" t="inlineStr"/>
@@ -43273,21 +43563,9 @@
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="D699" s="2" t="inlineStr">
-        <is>
-          <t>DOCTORA DE ALCALÁ 3 ALCALÁ DE HENARES</t>
-        </is>
-      </c>
-      <c r="E699" s="2" t="inlineStr">
-        <is>
-          <t>INSTALACIÓN ASCENSOR</t>
-        </is>
-      </c>
-      <c r="F699" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="D699" s="2" t="inlineStr"/>
+      <c r="E699" s="2" t="n"/>
+      <c r="F699" s="2" t="inlineStr"/>
       <c r="G699" s="2" t="inlineStr"/>
       <c r="H699" s="2" t="inlineStr">
         <is>
@@ -43300,14 +43578,10 @@
       <c r="L699" s="2" t="n"/>
       <c r="M699" s="2" t="n"/>
       <c r="N699" s="2" t="n"/>
-      <c r="O699" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
+      <c r="O699" s="2" t="n"/>
       <c r="P699" s="2" t="inlineStr">
         <is>
-          <t>1xm1Uk6BLN7KJfw8qV-YjwyUKpwrTeyEo-6-22H8AnDw</t>
+          <t>1aq8Zcs1OuAoJnBgccuy2QQqlWYkkeRvrusnfUEMY7qc</t>
         </is>
       </c>
       <c r="Q699" s="2" t="inlineStr"/>
@@ -43330,9 +43604,21 @@
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="D700" s="2" t="inlineStr"/>
-      <c r="E700" s="2" t="n"/>
-      <c r="F700" s="2" t="inlineStr"/>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>URBANIZACION LAS ANCLAS CALLE GALEON .PAREJA . GUADALAJARA</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REPARACION DE FACHADA , TECHO DE TERRAZAS E IMPERMIABILIZACION DE BORDE DE CUBIERTA </t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G700" s="2" t="inlineStr"/>
       <c r="H700" s="2" t="inlineStr">
         <is>
@@ -43345,8 +43631,16 @@
       <c r="L700" s="2" t="n"/>
       <c r="M700" s="2" t="n"/>
       <c r="N700" s="2" t="n"/>
-      <c r="O700" s="2" t="n"/>
-      <c r="P700" s="2" t="n"/>
+      <c r="O700" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P700" s="2" t="inlineStr">
+        <is>
+          <t>1gOauBU8GmZGpgWTBgr2STLw0a0ciSnvzEhi0-IaQqtM</t>
+        </is>
+      </c>
       <c r="Q700" s="2" t="inlineStr"/>
       <c r="R700" s="2" t="inlineStr"/>
       <c r="S700" s="4" t="inlineStr"/>
@@ -43431,12 +43725,12 @@
       </c>
       <c r="E702" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACCESIBILIDAD MEDIANTE RAMPA </t>
+          <t xml:space="preserve">SUBVENCIÓN ACCESIBILIDAD </t>
         </is>
       </c>
       <c r="F702" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G702" s="2" t="inlineStr"/>
@@ -43458,7 +43752,7 @@
       </c>
       <c r="P702" s="2" t="inlineStr">
         <is>
-          <t>1utd-mcXcLxbri9eipmUIksWi54Xe8xPvPqpy84SABQk</t>
+          <t>1tfxj4Zd1QZojCwiK2EN7Gbp7Me6GcyfTekno5mzPC80</t>
         </is>
       </c>
       <c r="Q702" s="2" t="inlineStr"/>
@@ -43545,12 +43839,12 @@
       </c>
       <c r="E704" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN DE ELEVADOR CON DERRIBO DE ESCALERA</t>
+          <t xml:space="preserve">SUBVENCIÓN ACCESIBILIDAD </t>
         </is>
       </c>
       <c r="F704" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G704" s="2" t="inlineStr"/>
@@ -43572,7 +43866,7 @@
       </c>
       <c r="P704" s="2" t="inlineStr">
         <is>
-          <t>1Vk2hdC-NB8h7fi_3yPbHCVY64jFZj2hAzrCHOeA_hd4</t>
+          <t>1SAurgUBJsABDRJwNnO_MzjUBzacb7YwJ7DEHZc7DeqU</t>
         </is>
       </c>
       <c r="Q704" s="2" t="inlineStr">
@@ -43661,8 +43955,16 @@
           <t>FERENC PUSKAS 28 MADRID</t>
         </is>
       </c>
-      <c r="E706" s="2" t="n"/>
-      <c r="F706" s="2" t="inlineStr"/>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>REDACCIÓN DE MEDICIONES Y PRESUPUESTO CIEGO</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO</t>
+        </is>
+      </c>
       <c r="G706" s="2" t="inlineStr"/>
       <c r="H706" s="2" t="inlineStr">
         <is>
@@ -43699,8 +44001,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O706" s="2" t="n"/>
-      <c r="P706" s="2" t="n"/>
+      <c r="O706" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P706" s="2" t="inlineStr">
+        <is>
+          <t>1P8eVu2miRH8GiKde_34-amTJF9bQU4V1XhuHFe6aol8</t>
+        </is>
+      </c>
       <c r="Q706" s="2" t="inlineStr">
         <is>
           <t>tanda1 135: RESUELTO LEYENDO: Bloque nuevo MEDICIONES Y CIEGO (Mónica, 6-oct).</t>
@@ -44273,12 +44583,12 @@
       </c>
       <c r="E716" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCIONES ACCESIBILIDAD Y EFICIENCIA ENERGÉTICA</t>
+          <t xml:space="preserve">SUBVENCIÓN EFICIENCIA ENERGÉTICA </t>
         </is>
       </c>
       <c r="F716" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G716" s="2" t="inlineStr"/>
@@ -44300,7 +44610,7 @@
       </c>
       <c r="P716" s="2" t="inlineStr">
         <is>
-          <t>158aSDqc1b1I2mpbpbVEXg4Q8koAyCWNm4aertcmiucs</t>
+          <t>1bs_ki35CBKfsKXkbW7Mr9DqEolbDgTgXmoSQHI5_22o</t>
         </is>
       </c>
       <c r="Q716" s="2" t="inlineStr"/>
@@ -44452,21 +44762,9 @@
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D719" s="2" t="inlineStr">
-        <is>
-          <t>VILLAFUERTE 23 MADRID</t>
-        </is>
-      </c>
-      <c r="E719" s="2" t="inlineStr">
-        <is>
-          <t>PLATAFORMA VERTICAL + BAJADA ASCENSORES A COTA GARAJE</t>
-        </is>
-      </c>
-      <c r="F719" s="2" t="inlineStr">
-        <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
-        </is>
-      </c>
+      <c r="D719" s="2" t="inlineStr"/>
+      <c r="E719" s="2" t="n"/>
+      <c r="F719" s="2" t="inlineStr"/>
       <c r="G719" s="2" t="inlineStr"/>
       <c r="H719" s="2" t="inlineStr">
         <is>
@@ -44479,14 +44777,10 @@
       <c r="L719" s="2" t="n"/>
       <c r="M719" s="2" t="n"/>
       <c r="N719" s="2" t="n"/>
-      <c r="O719" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="O719" s="2" t="n"/>
       <c r="P719" s="2" t="inlineStr">
         <is>
-          <t>1os5AWBo_dFeOAuRtSwFW9cyNSCma7xAX07KqJ2XYGKk</t>
+          <t>1aeDM9pBXxmiyBBJIm_JNlf3pzOdWSFj8KYnjtFLNHys</t>
         </is>
       </c>
       <c r="Q719" s="2" t="inlineStr"/>
@@ -44573,7 +44867,7 @@
       </c>
       <c r="E721" s="2" t="inlineStr">
         <is>
-          <t>PLATAFORMA VERTICAL + BAJADA ASCENSORES A COTA GARAJE</t>
+          <t xml:space="preserve">PLATAFORMA VERTICAL </t>
         </is>
       </c>
       <c r="F721" s="2" t="inlineStr">
@@ -44600,7 +44894,7 @@
       </c>
       <c r="P721" s="2" t="inlineStr">
         <is>
-          <t>1os5AWBo_dFeOAuRtSwFW9cyNSCma7xAX07KqJ2XYGKk</t>
+          <t>1X_ppje9xnwoXbghxefsYwVcp9W1O_hUkeKw6r-F4h1c</t>
         </is>
       </c>
       <c r="Q721" s="2" t="inlineStr"/>
@@ -44680,9 +44974,21 @@
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D723" s="2" t="inlineStr"/>
-      <c r="E723" s="2" t="n"/>
-      <c r="F723" s="2" t="inlineStr"/>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>ZAMORA 8 FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>REMODELACIÓN DE PORTAL</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G723" s="2" t="inlineStr"/>
       <c r="H723" s="2" t="inlineStr">
         <is>
@@ -44696,7 +45002,11 @@
       <c r="M723" s="2" t="n"/>
       <c r="N723" s="2" t="n"/>
       <c r="O723" s="2" t="n"/>
-      <c r="P723" s="2" t="n"/>
+      <c r="P723" s="2" t="inlineStr">
+        <is>
+          <t>1JevhAfFteoW-xf0-6IyIoobTUNsFak5cMjk22v4Fpx4</t>
+        </is>
+      </c>
       <c r="Q723" s="2" t="inlineStr"/>
       <c r="R723" s="2" t="inlineStr"/>
       <c r="S723" s="4" t="inlineStr"/>
@@ -44915,8 +45225,16 @@
           <t>CASTILLA LA NUEVA 37 BIS FUENLABRADA</t>
         </is>
       </c>
-      <c r="E727" s="2" t="n"/>
-      <c r="F727" s="2" t="inlineStr"/>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>SUBVENCIÓN ACCESIBILIDAD</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="inlineStr">
+        <is>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
+        </is>
+      </c>
       <c r="G727" s="2" t="inlineStr"/>
       <c r="H727" s="2" t="inlineStr">
         <is>
@@ -44954,8 +45272,16 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="O727" s="2" t="n"/>
-      <c r="P727" s="2" t="n"/>
+      <c r="O727" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P727" s="2" t="inlineStr">
+        <is>
+          <t>1fhWi7_9U_3DlPHZKHpKXwo11YK7fB3-KjFEZGN_Yy2U</t>
+        </is>
+      </c>
       <c r="Q727" s="2" t="inlineStr"/>
       <c r="R727" s="2" t="inlineStr"/>
       <c r="S727" s="4" t="inlineStr"/>
@@ -44988,7 +45314,7 @@
       </c>
       <c r="F728" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G728" s="2" t="inlineStr"/>
@@ -45010,7 +45336,7 @@
       </c>
       <c r="P728" s="2" t="inlineStr">
         <is>
-          <t>1ngQKWIh52j4t3ukO2loWnBbCY5gSVVZ2rPI7etTc_j4</t>
+          <t>1lwCDuXyHsGbb-nJJ_9myqablPN3UKNKpXW4EEE7gdHg</t>
         </is>
       </c>
       <c r="Q728" s="2" t="inlineStr">
@@ -45622,12 +45948,12 @@
       </c>
       <c r="E739" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F739" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G739" s="2" t="inlineStr"/>
@@ -45649,7 +45975,7 @@
       </c>
       <c r="P739" s="2" t="inlineStr">
         <is>
-          <t>1_6yJfYU3I8xhIzLBnKp4EJLg-JM-hMbKmAChclsNPfE</t>
+          <t>1YdabSYuZrNJMjjKh2KItaEnLE--w00ldMICT5KRWdwc</t>
         </is>
       </c>
       <c r="Q739" s="2" t="inlineStr"/>
@@ -45858,12 +46184,12 @@
       </c>
       <c r="E743" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENVOLVENTE TERMICA </t>
+          <t xml:space="preserve">SUBVENCIONES DE EFICIENCIA ENERGETICA </t>
         </is>
       </c>
       <c r="F743" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G743" s="2" t="inlineStr"/>
@@ -45885,7 +46211,7 @@
       </c>
       <c r="P743" s="2" t="inlineStr">
         <is>
-          <t>1UFRTN_NUdGjo8wzD6Q-rmKaaqWZ_RIoB2AFEcmzK3hM</t>
+          <t>1e75_K_X3mruQ65WiycDrPCs0MeUZI41SBh-y1FrrqfQ</t>
         </is>
       </c>
       <c r="Q743" s="2" t="inlineStr"/>
@@ -46037,7 +46363,7 @@
       </c>
       <c r="E746" s="2" t="inlineStr">
         <is>
-          <t>PROYECTO CONJUNTO ASCENSOR Y SATE</t>
+          <t xml:space="preserve">ENVOLVENTE TERMICA (SATE) </t>
         </is>
       </c>
       <c r="F746" s="2" t="inlineStr">
@@ -46064,7 +46390,7 @@
       </c>
       <c r="P746" s="2" t="inlineStr">
         <is>
-          <t>13QCKnA2Jng553Spp341X9Hknf3lRQKuoD2xY9LFJ3Ho</t>
+          <t>17uLm8v7e2cdju5o-l7fdNlbrOX7JJAbeMU3B_k7bflY</t>
         </is>
       </c>
       <c r="Q746" s="2" t="inlineStr">
@@ -46460,12 +46786,12 @@
       </c>
       <c r="E753" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENVOLVENTE TERMICA </t>
+          <t xml:space="preserve">SUBVENCIONES DE EFICIENCIA ENERGETICA </t>
         </is>
       </c>
       <c r="F753" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G753" s="2" t="inlineStr"/>
@@ -46487,7 +46813,7 @@
       </c>
       <c r="P753" s="2" t="inlineStr">
         <is>
-          <t>1L-ktLDamsW5_9euWGlYbIpMFjo-YSlQMwms1o6vFm3w</t>
+          <t>1ZQZlCLi41qZvTtEiRdUvYDGwLrjtFhRXJeixE2-qRRw</t>
         </is>
       </c>
       <c r="Q753" s="2" t="inlineStr"/>
@@ -46510,9 +46836,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="D754" s="2" t="inlineStr"/>
-      <c r="E754" s="2" t="n"/>
-      <c r="F754" s="2" t="inlineStr"/>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>SANTA SUSANA 41 MADRID</t>
+        </is>
+      </c>
+      <c r="E754" s="2" t="inlineStr">
+        <is>
+          <t>ENVOLVENTE TÉRMICA (SATE ) PARA FACHADA Y CUBIERTA</t>
+        </is>
+      </c>
+      <c r="F754" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS, IEE, LEE, CEE</t>
+        </is>
+      </c>
       <c r="G754" s="2" t="inlineStr"/>
       <c r="H754" s="2" t="inlineStr">
         <is>
@@ -46525,8 +46863,16 @@
       <c r="L754" s="2" t="n"/>
       <c r="M754" s="2" t="n"/>
       <c r="N754" s="2" t="n"/>
-      <c r="O754" s="2" t="n"/>
-      <c r="P754" s="2" t="n"/>
+      <c r="O754" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P754" s="2" t="inlineStr">
+        <is>
+          <t>1Kl0HTIwaUjoRFvKjoKDtNPEwHEeMyNbnKeHuN1oScnY</t>
+        </is>
+      </c>
       <c r="Q754" s="2" t="inlineStr"/>
       <c r="R754" s="2" t="inlineStr"/>
       <c r="S754" s="4" t="inlineStr"/>
@@ -46668,12 +47014,12 @@
       </c>
       <c r="E757" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENVOLVENTE TERMICA (SATE) </t>
+          <t xml:space="preserve">SUBVENCIONES DE EFICIENCIA ENERGETICA </t>
         </is>
       </c>
       <c r="F757" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G757" s="2" t="inlineStr"/>
@@ -46695,7 +47041,7 @@
       </c>
       <c r="P757" s="2" t="inlineStr">
         <is>
-          <t>1tAPtR3la4S4mwGMYmXUfZ3XQRsYjUD96zfaSxJNFJE4</t>
+          <t>1JF5HKE14P6jdNBMajDz6WP0yc34O2mNBOFm7EL9Rvhs</t>
         </is>
       </c>
       <c r="Q757" s="2" t="inlineStr"/>
@@ -46797,9 +47143,21 @@
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="D759" s="2" t="inlineStr"/>
-      <c r="E759" s="2" t="n"/>
-      <c r="F759" s="2" t="inlineStr"/>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>PLAZA MALICIOSA 4-5 MADRID</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENVOLVENTE TERMICA (SATE) </t>
+        </is>
+      </c>
+      <c r="F759" s="2" t="inlineStr">
+        <is>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+        </is>
+      </c>
       <c r="G759" s="2" t="inlineStr"/>
       <c r="H759" s="2" t="inlineStr">
         <is>
@@ -46812,8 +47170,16 @@
       <c r="L759" s="2" t="n"/>
       <c r="M759" s="2" t="n"/>
       <c r="N759" s="2" t="n"/>
-      <c r="O759" s="2" t="n"/>
-      <c r="P759" s="2" t="n"/>
+      <c r="O759" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P759" s="2" t="inlineStr">
+        <is>
+          <t>1tAPtR3la4S4mwGMYmXUfZ3XQRsYjUD96zfaSxJNFJE4</t>
+        </is>
+      </c>
       <c r="Q759" s="2" t="inlineStr"/>
       <c r="R759" s="2" t="inlineStr"/>
       <c r="S759" s="4" t="inlineStr"/>
@@ -46955,12 +47321,12 @@
       </c>
       <c r="E762" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ELEVADOR</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F762" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G762" s="2" t="inlineStr"/>
@@ -46982,7 +47348,7 @@
       </c>
       <c r="P762" s="2" t="inlineStr">
         <is>
-          <t>15TsYmLbLjxKGMQLBGi9D7nw_M_okCrxPKhGdW8ToCuI</t>
+          <t>1dfU1yAV9Y_qnGowT1A6PZhnPOOmluNwm1SQEicFEssc</t>
         </is>
       </c>
       <c r="Q762" s="2" t="inlineStr"/>
@@ -47126,12 +47492,12 @@
       </c>
       <c r="E765" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F765" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G765" s="2" t="inlineStr"/>
@@ -47153,7 +47519,7 @@
       </c>
       <c r="P765" s="2" t="inlineStr">
         <is>
-          <t>1S92aosMPTlZ0mTyITuEAFR12yQsVGW8cdHHoUfiAsm4</t>
+          <t>1DxbpEMb5WNh6T6Icd8c9zkKfy69amOJ1Bn5_OlE5D3M</t>
         </is>
       </c>
       <c r="Q765" s="2" t="inlineStr"/>
@@ -47297,12 +47663,12 @@
       </c>
       <c r="E768" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBVENCIONES DE EFICIENCIA ENERGETICA </t>
+          <t>INSTALACIÓN ASCENSOR</t>
         </is>
       </c>
       <c r="F768" s="2" t="inlineStr">
         <is>
-          <t>TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
+          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
         </is>
       </c>
       <c r="G768" s="2" t="inlineStr"/>
@@ -47324,7 +47690,7 @@
       </c>
       <c r="P768" s="2" t="inlineStr">
         <is>
-          <t>160VamawGVJeVaH1dQloMIABt30B4RUe-FJ8yN8BWBw4</t>
+          <t>15siuRuu7quzEr3KWtuqjwHXWiugrv1mWJneWoMjVW-A</t>
         </is>
       </c>
       <c r="Q768" s="2" t="inlineStr"/>
@@ -47411,7 +47777,7 @@
       </c>
       <c r="E770" s="2" t="inlineStr">
         <is>
-          <t>PROYECTO CONJUNTO DE SATE Y ASCENSOR</t>
+          <t>ENVOLVENTE TERMICA (SATE EN CUBIERTA Y FACHADA )</t>
         </is>
       </c>
       <c r="F770" s="2" t="inlineStr">
@@ -47438,7 +47804,7 @@
       </c>
       <c r="P770" s="2" t="inlineStr">
         <is>
-          <t>1tOlOtAHfTtxZdoYoNogqm16AvDR6D_rgH3vT3hpx1EQ</t>
+          <t>1mgbriBdW54YwxNlwKG_YYRHnNClHyBQQeqPdeYkp2Kg</t>
         </is>
       </c>
       <c r="Q770" s="2" t="inlineStr"/>
@@ -47468,12 +47834,12 @@
       </c>
       <c r="E771" s="2" t="inlineStr">
         <is>
-          <t>PROYECTO CONJUNTO DE SATE Y ASCENSOR</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F771" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G771" s="2" t="inlineStr"/>
@@ -47495,7 +47861,7 @@
       </c>
       <c r="P771" s="2" t="inlineStr">
         <is>
-          <t>1tOlOtAHfTtxZdoYoNogqm16AvDR6D_rgH3vT3hpx1EQ</t>
+          <t>17gq8SpOOxSA7qM01k1fmo6lEmCOn2bNFpb69jNiQPo4</t>
         </is>
       </c>
       <c r="Q771" s="2" t="inlineStr"/>
@@ -47525,12 +47891,12 @@
       </c>
       <c r="E772" s="2" t="inlineStr">
         <is>
-          <t>PROYECTO CONJUNTO DE SATE Y ASCENSOR</t>
+          <t xml:space="preserve">SUBVENCIONES DE EFICIENCIA ENERGETICA Y ACCESIBILIDAD </t>
         </is>
       </c>
       <c r="F772" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, TRAMITACION SUBVENCIONES EFICIENCIA ENERGETICA, IEE, LEE, CEE</t>
         </is>
       </c>
       <c r="G772" s="2" t="inlineStr"/>
@@ -47552,7 +47918,7 @@
       </c>
       <c r="P772" s="2" t="inlineStr">
         <is>
-          <t>1tOlOtAHfTtxZdoYoNogqm16AvDR6D_rgH3vT3hpx1EQ</t>
+          <t>1uUWN5qHuA3XKJpzJ85cGKnnTU6yOQ4cFATsncEvoV1Y</t>
         </is>
       </c>
       <c r="Q772" s="2" t="inlineStr"/>
@@ -47810,12 +48176,12 @@
       </c>
       <c r="E777" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR Y PLATAFORMA ELEVADORA VERTICAL</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F777" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G777" s="2" t="inlineStr"/>
@@ -47837,7 +48203,7 @@
       </c>
       <c r="P777" s="2" t="inlineStr">
         <is>
-          <t>167-Et0Aie6M59MvTXObS2ZGz1LXO9hSVKmZ0bz4ZUEY</t>
+          <t>1AQ_A_zSIv0khFEbN1FQi64jtcELIbch84ygUzffnOfQ</t>
         </is>
       </c>
       <c r="Q777" s="2" t="inlineStr"/>
@@ -47924,12 +48290,12 @@
       </c>
       <c r="E779" s="2" t="inlineStr">
         <is>
-          <t>INSTALACIÓN ASCENSOR</t>
+          <t>SUBVENCIONES ACCESIBILIDAD</t>
         </is>
       </c>
       <c r="F779" s="2" t="inlineStr">
         <is>
-          <t>TOMA DE DATOS Y MODELADO 3D, REDACCION PROYECTO, TRAMITACION LICENCIAS, TRAMITACION 3 PRESUPUESTOS, CERTIFICADO FIN DE OBRA, DF, CSS</t>
+          <t>TRAMITACION SUBVENCIONES ACCESIBILIDAD, IEE, CEE</t>
         </is>
       </c>
       <c r="G779" s="2" t="inlineStr"/>
@@ -47951,7 +48317,7 @@
       </c>
       <c r="P779" s="2" t="inlineStr">
         <is>
-          <t>1bC0qhOKYUF9Y-wxMeSj2OQnzpr3F9W4kGoJFeeoUSD0</t>
+          <t>1C-aB8GtWIZhKepvnWP0snbE-mOvIwXtK-RKI5DeS29g</t>
         </is>
       </c>
       <c r="Q779" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Ayamonte 2: sustituida por rebaja de alcance (todo -> solo cubierta)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/manifiesto_hojas_2026.xlsx
+++ b/docs/manifiesto_hojas_2026.xlsx
@@ -8019,9 +8019,9 @@
           <t>HE-2026-0115</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
-        <is>
-          <t>ENVIADA SIN FIRMAR</t>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>SUSTITUIDA</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -8068,8 +8068,9 @@
       </c>
       <c r="Q116" s="2" t="inlineStr">
         <is>
-          <t>hoja distinta, no versión (leído): Objetos distintos: la del 10-02 es proyecto de envolvente térmica (SATE con cesión de CAES, 18.220) y la del 16-02 es proyecto de cubierta (7.000); la firmada es la de cubierta.
-PARA TI · ¿sustituida por una posterior?: La antigua es proyecto SATE de fachada + subvención EE con CAES; las posteriores son proyecto de CUBIERTA y subvención de ACCESIBILIDAD (que casa con la hoja ASC2), ninguna recoge el SATE: puede que lo cambiaran por cubierta o que siga aparte.</t>
+          <t>PARA TI · ¿sustituida por una posterior?: La antigua es proyecto SATE de fachada + subvención EE con CAES; las posteriores son proyecto de CUBIERTA y subvención de ACCESIBILIDAD (que casa con la hoja ASC2), ninguna recoge el SATE: puede que lo cambiaran por cubierta o que siga aparte.
+SUSTITUIDA: Rebaja de alcance: primero lo querían todo (SATE + subvención con CAES) y luego solo cubierta, porque les salía caro. Negociación habitual (Mónica).
+sustituida por: HE-2026-0136, HE-2026-0137</t>
         </is>
       </c>
       <c r="R116" s="2" t="inlineStr"/>
@@ -9326,7 +9327,11 @@
           <t>1xQ9da0evJK54LFtz6v5Ia8NnBuICWYqS4UaJMydcrqA</t>
         </is>
       </c>
-      <c r="Q137" s="2" t="inlineStr"/>
+      <c r="Q137" s="2" t="inlineStr">
+        <is>
+          <t>sustituye a la(s) hoja(s) anterior(es): Rebaja de alcance: primero lo querían todo (SATE + subvención con CAES) y luego solo cubierta, porque les salía caro. Negociación habitual (Mónica).</t>
+        </is>
+      </c>
       <c r="R137" s="2" t="inlineStr"/>
       <c r="S137" s="4" t="inlineStr"/>
     </row>
@@ -9413,7 +9418,7 @@
       </c>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t>hoja distinta, no versión (leído): Objetos distintos: la del 10-02 es proyecto de envolvente térmica (SATE con cesión de CAES, 18.220) y la del 16-02 es proyecto de cubierta (7.000); la firmada es la de cubierta.</t>
+          <t>sustituye a la(s) hoja(s) anterior(es): Rebaja de alcance: primero lo querían todo (SATE + subvención con CAES) y luego solo cubierta, porque les salía caro. Negociación habitual (Mónica).</t>
         </is>
       </c>
       <c r="R138" s="2" t="inlineStr"/>

</xml_diff>